<commit_message>
EPBDS-14250 Drop 'cacheable' property support
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules/doc/TablePropertyDefinition.xlsx
+++ b/DEV/org.openl.rules/doc/TablePropertyDefinition.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="283">
   <si>
     <t>Display Name</t>
   </si>
@@ -696,15 +696,6 @@
   </si>
   <si>
     <t>The name of the package for spreadsheet result beans generation</t>
-  </si>
-  <si>
-    <t>Cacheable</t>
-  </si>
-  <si>
-    <t>cacheable</t>
-  </si>
-  <si>
-    <t>Defines whether or not to use cache while recalculating the table for a variation, depending on the rule input</t>
   </si>
   <si>
     <t>Empty Result Processing</t>
@@ -941,7 +932,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color indexed="10"/>
+      <color indexed="9"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -954,7 +945,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="10"/>
+        <fgColor indexed="9"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -993,28 +984,28 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
         <color indexed="8"/>
@@ -1023,16 +1014,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
         <color indexed="8"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1056,13 +1047,13 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1074,10 +1065,10 @@
         <color indexed="8"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1089,10 +1080,10 @@
         <color indexed="8"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1101,37 +1092,37 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
         <color indexed="8"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
         <color indexed="8"/>
@@ -1143,13 +1134,13 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="medium">
         <color indexed="8"/>
@@ -1158,16 +1149,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="medium">
         <color indexed="8"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1221,13 +1212,13 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1402,20 +1393,20 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1451,11 +1442,8 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
@@ -1463,6 +1451,9 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
@@ -1484,6 +1475,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
@@ -1532,10 +1529,10 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1547,7 +1544,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1565,7 +1562,7 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="22" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1603,8 +1600,8 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffff0000"/>
       <rgbColor rgb="ff4f81bd"/>
       <rgbColor rgb="ffb7dee8"/>
@@ -1760,9 +1757,9 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -1842,7 +1839,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1870,10 +1867,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2129,9 +2126,9 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
             <a:srgbClr val="000000">
-              <a:alpha val="38000"/>
+              <a:alpha val="35000"/>
             </a:srgbClr>
           </a:outerShdw>
         </a:effectLst>
@@ -2419,7 +2416,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -2447,10 +2444,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2969,34 +2966,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:ALL67"/>
+  <dimension ref="A1:T66"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.85156" style="16" customWidth="1"/>
-    <col min="2" max="2" width="17.5" style="16" customWidth="1"/>
-    <col min="3" max="3" width="15" style="16" customWidth="1"/>
-    <col min="4" max="4" width="12.5" style="16" customWidth="1"/>
-    <col min="5" max="5" width="18.5" style="16" customWidth="1"/>
-    <col min="6" max="6" width="19.1719" style="16" customWidth="1"/>
-    <col min="7" max="7" width="20.8516" style="16" customWidth="1"/>
-    <col min="8" max="8" width="11.3516" style="16" customWidth="1"/>
-    <col min="9" max="9" width="22" style="16" customWidth="1"/>
-    <col min="10" max="10" width="22.5" style="16" customWidth="1"/>
-    <col min="11" max="11" width="8.35156" style="16" customWidth="1"/>
-    <col min="12" max="12" width="38.8516" style="16" customWidth="1"/>
-    <col min="13" max="13" width="49.8516" style="16" customWidth="1"/>
-    <col min="14" max="14" width="20.1719" style="16" customWidth="1"/>
-    <col min="15" max="15" width="33" style="16" customWidth="1"/>
-    <col min="16" max="16" width="8.5" style="16" customWidth="1"/>
-    <col min="17" max="17" width="12.5" style="16" customWidth="1"/>
-    <col min="18" max="18" width="11.8516" style="16" customWidth="1"/>
-    <col min="19" max="19" width="25.6719" style="16" customWidth="1"/>
-    <col min="20" max="20" width="73.3516" style="16" customWidth="1"/>
-    <col min="21" max="1000" width="8.85156" style="16" customWidth="1"/>
-    <col min="1001" max="16384" width="8.85156" style="15" customWidth="1"/>
+    <col min="1" max="1" width="8.85156" style="15" customWidth="1"/>
+    <col min="2" max="2" width="17.5" style="15" customWidth="1"/>
+    <col min="3" max="3" width="15" style="15" customWidth="1"/>
+    <col min="4" max="4" width="12.5" style="15" customWidth="1"/>
+    <col min="5" max="5" width="18.5" style="15" customWidth="1"/>
+    <col min="6" max="6" width="19.1719" style="15" customWidth="1"/>
+    <col min="7" max="7" width="20.8516" style="15" customWidth="1"/>
+    <col min="8" max="8" width="11.3516" style="15" customWidth="1"/>
+    <col min="9" max="9" width="22" style="15" customWidth="1"/>
+    <col min="10" max="10" width="22.5" style="15" customWidth="1"/>
+    <col min="11" max="11" width="8.35156" style="15" customWidth="1"/>
+    <col min="12" max="12" width="38.8516" style="15" customWidth="1"/>
+    <col min="13" max="13" width="49.8516" style="15" customWidth="1"/>
+    <col min="14" max="14" width="20.1719" style="15" customWidth="1"/>
+    <col min="15" max="15" width="33" style="15" customWidth="1"/>
+    <col min="16" max="16" width="8.5" style="15" customWidth="1"/>
+    <col min="17" max="17" width="12.5" style="15" customWidth="1"/>
+    <col min="18" max="18" width="11.8516" style="15" customWidth="1"/>
+    <col min="19" max="19" width="25.6719" style="15" customWidth="1"/>
+    <col min="20" max="20" width="73.3516" style="15" customWidth="1"/>
+    <col min="21" max="16384" width="8.85156" style="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="17" customFormat="1" ht="11.25" customHeight="1">
+    <row r="1" ht="11.25" customHeight="1">
+      <c r="A1" s="16"/>
       <c r="B1" t="s" s="5">
         <v>0</v>
       </c>
@@ -3012,8 +3009,17 @@
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
       <c r="L1" s="7"/>
-    </row>
-    <row r="2" s="17" customFormat="1" ht="11.25" customHeight="1">
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+    </row>
+    <row r="2" ht="11.25" customHeight="1">
+      <c r="A2" s="16"/>
       <c r="B2" t="s" s="5">
         <v>2</v>
       </c>
@@ -3029,16 +3035,43 @@
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
-    </row>
-    <row r="3" s="17" customFormat="1" ht="57.75" customHeight="1">
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="9"/>
+    </row>
+    <row r="3" ht="57.75" customHeight="1">
+      <c r="A3" s="16"/>
       <c r="B3" t="s" s="5">
         <v>4</v>
       </c>
       <c r="C3" t="s" s="8">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" s="17" customFormat="1" ht="22.5" customHeight="1">
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="16"/>
       <c r="B4" t="s" s="5">
         <v>6</v>
       </c>
@@ -3054,8 +3087,17 @@
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
-    </row>
-    <row r="5" s="17" customFormat="1" ht="22.5" customHeight="1">
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="16"/>
       <c r="B5" t="s" s="5">
         <v>8</v>
       </c>
@@ -3071,24 +3113,69 @@
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
-    </row>
-    <row r="6" s="17" customFormat="1" ht="51.75" customHeight="1">
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="9"/>
+    </row>
+    <row r="6" ht="51.75" customHeight="1">
+      <c r="A6" s="16"/>
       <c r="B6" t="s" s="5">
         <v>10</v>
       </c>
       <c r="C6" t="s" s="8">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" s="17" customFormat="1" ht="42.75" customHeight="1">
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+    </row>
+    <row r="7" ht="42.75" customHeight="1">
+      <c r="A7" s="16"/>
       <c r="B7" t="s" s="5">
         <v>12</v>
       </c>
       <c r="C7" t="s" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" s="17" customFormat="1" ht="33" customHeight="1">
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="9"/>
+      <c r="T7" s="9"/>
+    </row>
+    <row r="8" ht="33" customHeight="1">
+      <c r="A8" s="16"/>
       <c r="B8" t="s" s="5">
         <v>14</v>
       </c>
@@ -3104,8 +3191,17 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-    </row>
-    <row r="9" s="17" customFormat="1" ht="33" customHeight="1">
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+    </row>
+    <row r="9" ht="33" customHeight="1">
+      <c r="A9" s="16"/>
       <c r="B9" t="s" s="5">
         <v>16</v>
       </c>
@@ -3121,17 +3217,39 @@
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
-    </row>
-    <row r="10" s="17" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B10" s="18"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-    </row>
-    <row r="11" s="17" customFormat="1" ht="15" customHeight="1">
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="9"/>
+      <c r="T9" s="9"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="9"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="16"/>
       <c r="B11" t="s" s="20">
         <v>27</v>
       </c>
@@ -3154,7 +3272,8 @@
       <c r="S11" s="21"/>
       <c r="T11" s="21"/>
     </row>
-    <row r="12" s="17" customFormat="1" ht="45" customHeight="1">
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="16"/>
       <c r="B12" t="s" s="22">
         <v>28</v>
       </c>
@@ -3213,7 +3332,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" s="17" customFormat="1" ht="38.25" customHeight="1">
+    <row r="13" ht="38.25" customHeight="1">
+      <c r="A13" s="16"/>
       <c r="B13" t="s" s="22">
         <v>0</v>
       </c>
@@ -3272,7 +3392,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="16"/>
       <c r="B14" t="s" s="23">
         <v>2</v>
       </c>
@@ -3319,7 +3440,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="16"/>
       <c r="B15" t="s" s="23">
         <v>66</v>
       </c>
@@ -3362,7 +3484,8 @@
         <v>70</v>
       </c>
     </row>
-    <row r="16" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="16"/>
       <c r="B16" t="s" s="23">
         <v>71</v>
       </c>
@@ -3409,7 +3532,8 @@
         <v>76</v>
       </c>
     </row>
-    <row r="17" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="16"/>
       <c r="B17" t="s" s="23">
         <v>77</v>
       </c>
@@ -3458,7 +3582,8 @@
         <v>82</v>
       </c>
     </row>
-    <row r="18" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="16"/>
       <c r="B18" t="s" s="23">
         <v>83</v>
       </c>
@@ -3505,7 +3630,8 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="16"/>
       <c r="B19" t="s" s="23">
         <v>87</v>
       </c>
@@ -3554,7 +3680,8 @@
         <v>89</v>
       </c>
     </row>
-    <row r="20" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="16"/>
       <c r="B20" t="s" s="23">
         <v>24</v>
       </c>
@@ -3597,7 +3724,8 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="16"/>
       <c r="B21" t="s" s="23">
         <v>91</v>
       </c>
@@ -3640,7 +3768,8 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="16"/>
       <c r="B22" t="s" s="23">
         <v>95</v>
       </c>
@@ -3689,7 +3818,8 @@
         <v>102</v>
       </c>
     </row>
-    <row r="23" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="16"/>
       <c r="B23" t="s" s="23">
         <v>103</v>
       </c>
@@ -3738,7 +3868,8 @@
         <v>107</v>
       </c>
     </row>
-    <row r="24" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="16"/>
       <c r="B24" t="s" s="23">
         <v>108</v>
       </c>
@@ -3787,7 +3918,8 @@
         <v>112</v>
       </c>
     </row>
-    <row r="25" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="16"/>
       <c r="B25" t="s" s="23">
         <v>113</v>
       </c>
@@ -3836,7 +3968,8 @@
         <v>117</v>
       </c>
     </row>
-    <row r="26" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="16"/>
       <c r="B26" t="s" s="23">
         <v>118</v>
       </c>
@@ -3881,7 +4014,8 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="16"/>
       <c r="B27" t="s" s="23">
         <v>123</v>
       </c>
@@ -3926,7 +4060,8 @@
         <v>127</v>
       </c>
     </row>
-    <row r="28" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="16"/>
       <c r="B28" t="s" s="23">
         <v>128</v>
       </c>
@@ -3971,7 +4106,8 @@
         <v>132</v>
       </c>
     </row>
-    <row r="29" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="16"/>
       <c r="B29" t="s" s="23">
         <v>133</v>
       </c>
@@ -4016,7 +4152,8 @@
         <v>137</v>
       </c>
     </row>
-    <row r="30" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="16"/>
       <c r="B30" t="s" s="23">
         <v>138</v>
       </c>
@@ -4061,7 +4198,8 @@
         <v>142</v>
       </c>
     </row>
-    <row r="31" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="16"/>
       <c r="B31" t="s" s="23">
         <v>143</v>
       </c>
@@ -4106,7 +4244,8 @@
         <v>147</v>
       </c>
     </row>
-    <row r="32" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="16"/>
       <c r="B32" t="s" s="23">
         <v>148</v>
       </c>
@@ -4153,7 +4292,8 @@
         <v>152</v>
       </c>
     </row>
-    <row r="33" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="16"/>
       <c r="B33" t="s" s="23">
         <v>153</v>
       </c>
@@ -4196,7 +4336,8 @@
         <v>156</v>
       </c>
     </row>
-    <row r="34" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="16"/>
       <c r="B34" t="s" s="23">
         <v>157</v>
       </c>
@@ -4241,7 +4382,8 @@
         <v>161</v>
       </c>
     </row>
-    <row r="35" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="16"/>
       <c r="B35" t="s" s="23">
         <v>162</v>
       </c>
@@ -4286,7 +4428,8 @@
         <v>166</v>
       </c>
     </row>
-    <row r="36" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="16"/>
       <c r="B36" t="s" s="23">
         <v>167</v>
       </c>
@@ -4327,7 +4470,8 @@
         <v>171</v>
       </c>
     </row>
-    <row r="37" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="16"/>
       <c r="B37" t="s" s="23">
         <v>172</v>
       </c>
@@ -4355,7 +4499,7 @@
         <v>169</v>
       </c>
       <c r="N37" t="b" s="26">
-        <f t="shared" si="0" ref="N37:N51">TRUE()</f>
+        <f t="shared" si="0" ref="N37:N50">TRUE()</f>
         <v>1</v>
       </c>
       <c r="O37" t="s" s="23">
@@ -4371,7 +4515,8 @@
         <v>176</v>
       </c>
     </row>
-    <row r="38" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="16"/>
       <c r="B38" t="s" s="23">
         <v>177</v>
       </c>
@@ -4418,7 +4563,8 @@
         <v>182</v>
       </c>
     </row>
-    <row r="39" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="16"/>
       <c r="B39" t="s" s="23">
         <v>183</v>
       </c>
@@ -4461,7 +4607,8 @@
         <v>186</v>
       </c>
     </row>
-    <row r="40" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="16"/>
       <c r="B40" t="s" s="23">
         <v>187</v>
       </c>
@@ -4504,7 +4651,8 @@
         <v>191</v>
       </c>
     </row>
-    <row r="41" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="16"/>
       <c r="B41" t="s" s="23">
         <v>192</v>
       </c>
@@ -4532,7 +4680,7 @@
         <v>190</v>
       </c>
       <c r="N41" t="b" s="26">
-        <f t="shared" si="1" ref="N41:N52">FALSE()</f>
+        <f t="shared" si="1" ref="N41:N51">FALSE()</f>
         <v>0</v>
       </c>
       <c r="O41" s="24"/>
@@ -4546,7 +4694,8 @@
         <v>194</v>
       </c>
     </row>
-    <row r="42" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="16"/>
       <c r="B42" t="s" s="23">
         <v>195</v>
       </c>
@@ -4587,7 +4736,8 @@
         <v>200</v>
       </c>
     </row>
-    <row r="43" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="16"/>
       <c r="B43" t="s" s="23">
         <v>201</v>
       </c>
@@ -4630,7 +4780,8 @@
         <v>205</v>
       </c>
     </row>
-    <row r="44" s="17" customFormat="1" ht="32" customHeight="1">
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="16"/>
       <c r="B44" t="s" s="23">
         <v>206</v>
       </c>
@@ -4673,7 +4824,8 @@
         <v>212</v>
       </c>
     </row>
-    <row r="45" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="16"/>
       <c r="B45" t="s" s="23">
         <v>213</v>
       </c>
@@ -4716,7 +4868,8 @@
         <v>216</v>
       </c>
     </row>
-    <row r="46" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="16"/>
       <c r="B46" t="s" s="23">
         <v>217</v>
       </c>
@@ -4727,7 +4880,7 @@
         <v>58</v>
       </c>
       <c r="E46" t="s" s="23">
-        <v>174</v>
+        <v>219</v>
       </c>
       <c r="F46" s="24"/>
       <c r="G46" t="s" s="23">
@@ -4743,9 +4896,11 @@
       </c>
       <c r="L46" s="24"/>
       <c r="M46" t="s" s="23">
-        <v>99</v>
-      </c>
-      <c r="N46" s="24"/>
+        <v>190</v>
+      </c>
+      <c r="N46" t="s" s="23">
+        <v>220</v>
+      </c>
       <c r="O46" s="24"/>
       <c r="P46" s="24"/>
       <c r="Q46" s="24"/>
@@ -4754,21 +4909,20 @@
         <v>101</v>
       </c>
       <c r="T46" t="s" s="23">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="47" s="17" customFormat="1" ht="30" customHeight="1">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="16"/>
       <c r="B47" t="s" s="23">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C47" t="s" s="23">
-        <v>221</v>
-      </c>
-      <c r="D47" t="s" s="23">
-        <v>58</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="D47" s="24"/>
       <c r="E47" t="s" s="23">
-        <v>222</v>
+        <v>59</v>
       </c>
       <c r="F47" s="24"/>
       <c r="G47" t="s" s="23">
@@ -4784,12 +4938,12 @@
       </c>
       <c r="L47" s="24"/>
       <c r="M47" t="s" s="23">
-        <v>190</v>
-      </c>
-      <c r="N47" t="s" s="23">
-        <v>223</v>
-      </c>
-      <c r="O47" s="24"/>
+        <v>224</v>
+      </c>
+      <c r="N47" s="24"/>
+      <c r="O47" t="s" s="23">
+        <v>225</v>
+      </c>
       <c r="P47" s="24"/>
       <c r="Q47" s="24"/>
       <c r="R47" s="24"/>
@@ -4797,19 +4951,22 @@
         <v>101</v>
       </c>
       <c r="T47" t="s" s="23">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="48" s="17" customFormat="1" ht="30" customHeight="1">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="16"/>
       <c r="B48" t="s" s="23">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C48" t="s" s="23">
-        <v>226</v>
-      </c>
-      <c r="D48" s="24"/>
+        <v>228</v>
+      </c>
+      <c r="D48" t="s" s="23">
+        <v>58</v>
+      </c>
       <c r="E48" t="s" s="23">
-        <v>59</v>
+        <v>174</v>
       </c>
       <c r="F48" s="24"/>
       <c r="G48" t="s" s="23">
@@ -4823,14 +4980,17 @@
       <c r="K48" t="s" s="23">
         <v>58</v>
       </c>
-      <c r="L48" s="24"/>
+      <c r="L48" t="s" s="23">
+        <v>58</v>
+      </c>
       <c r="M48" t="s" s="23">
-        <v>227</v>
-      </c>
-      <c r="N48" s="24"/>
-      <c r="O48" t="s" s="23">
-        <v>228</v>
-      </c>
+        <v>229</v>
+      </c>
+      <c r="N48" t="b" s="26">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="O48" s="24"/>
       <c r="P48" s="24"/>
       <c r="Q48" s="24"/>
       <c r="R48" s="24"/>
@@ -4838,15 +4998,16 @@
         <v>101</v>
       </c>
       <c r="T48" t="s" s="23">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="49" s="17" customFormat="1" ht="30" customHeight="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="16"/>
       <c r="B49" t="s" s="23">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C49" t="s" s="23">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D49" t="s" s="23">
         <v>58</v>
@@ -4870,11 +5031,11 @@
         <v>58</v>
       </c>
       <c r="M49" t="s" s="23">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="N49" t="b" s="26">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="O49" s="24"/>
       <c r="P49" s="24"/>
@@ -4887,7 +5048,8 @@
         <v>233</v>
       </c>
     </row>
-    <row r="50" s="17" customFormat="1" ht="30" customHeight="1">
+    <row r="50" ht="31.5" customHeight="1">
+      <c r="A50" s="16"/>
       <c r="B50" t="s" s="23">
         <v>234</v>
       </c>
@@ -4916,7 +5078,7 @@
         <v>58</v>
       </c>
       <c r="M50" t="s" s="23">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="N50" t="b" s="26">
         <f t="shared" si="0"/>
@@ -4933,7 +5095,8 @@
         <v>236</v>
       </c>
     </row>
-    <row r="51" s="17" customFormat="1" ht="31.5" customHeight="1">
+    <row r="51" ht="32" customHeight="1">
+      <c r="A51" s="16"/>
       <c r="B51" t="s" s="23">
         <v>237</v>
       </c>
@@ -4962,11 +5125,11 @@
         <v>58</v>
       </c>
       <c r="M51" t="s" s="23">
-        <v>232</v>
+        <v>99</v>
       </c>
       <c r="N51" t="b" s="26">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="O51" s="24"/>
       <c r="P51" s="24"/>
@@ -4979,7 +5142,8 @@
         <v>239</v>
       </c>
     </row>
-    <row r="52" s="17" customFormat="1" ht="32" customHeight="1">
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="16"/>
       <c r="B52" t="s" s="23">
         <v>240</v>
       </c>
@@ -4990,14 +5154,16 @@
         <v>58</v>
       </c>
       <c r="E52" t="s" s="23">
-        <v>174</v>
-      </c>
-      <c r="F52" s="24"/>
+        <v>59</v>
+      </c>
+      <c r="F52" t="s" s="23">
+        <v>242</v>
+      </c>
       <c r="G52" t="s" s="23">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="H52" t="s" s="23">
-        <v>179</v>
+        <v>98</v>
       </c>
       <c r="I52" s="24"/>
       <c r="J52" s="24"/>
@@ -5005,16 +5171,15 @@
         <v>58</v>
       </c>
       <c r="L52" t="s" s="23">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="M52" t="s" s="23">
         <v>99</v>
       </c>
-      <c r="N52" t="b" s="26">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O52" s="24"/>
+      <c r="N52" s="24"/>
+      <c r="O52" t="s" s="23">
+        <v>243</v>
+      </c>
       <c r="P52" s="24"/>
       <c r="Q52" s="24"/>
       <c r="R52" s="24"/>
@@ -5022,151 +5187,363 @@
         <v>101</v>
       </c>
       <c r="T52" t="s" s="23">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="53" s="17" customFormat="1" ht="32" customHeight="1">
-      <c r="B53" t="s" s="23">
-        <v>243</v>
-      </c>
-      <c r="C53" t="s" s="23">
         <v>244</v>
       </c>
-      <c r="D53" t="s" s="23">
-        <v>58</v>
-      </c>
-      <c r="E53" t="s" s="23">
-        <v>59</v>
-      </c>
-      <c r="F53" t="s" s="23">
+    </row>
+    <row r="53" ht="13.55" customHeight="1">
+      <c r="A53" s="9"/>
+      <c r="B53" s="27"/>
+      <c r="C53" s="27"/>
+      <c r="D53" s="27"/>
+      <c r="E53" s="27"/>
+      <c r="F53" s="27"/>
+      <c r="G53" s="27"/>
+      <c r="H53" s="27"/>
+      <c r="I53" s="27"/>
+      <c r="J53" s="27"/>
+      <c r="K53" s="27"/>
+      <c r="L53" s="27"/>
+      <c r="M53" s="27"/>
+      <c r="N53" s="27"/>
+      <c r="O53" s="27"/>
+      <c r="P53" s="27"/>
+      <c r="Q53" s="27"/>
+      <c r="R53" s="27"/>
+      <c r="S53" s="27"/>
+      <c r="T53" s="27"/>
+    </row>
+    <row r="54" ht="13.55" customHeight="1">
+      <c r="A54" s="9"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="9"/>
+      <c r="I54" s="9"/>
+      <c r="J54" s="9"/>
+      <c r="K54" s="9"/>
+      <c r="L54" s="9"/>
+      <c r="M54" s="9"/>
+      <c r="N54" s="9"/>
+      <c r="O54" s="9"/>
+      <c r="P54" s="9"/>
+      <c r="Q54" s="9"/>
+      <c r="R54" s="9"/>
+      <c r="S54" s="9"/>
+      <c r="T54" s="9"/>
+    </row>
+    <row r="55" ht="13.55" customHeight="1">
+      <c r="A55" s="9"/>
+      <c r="B55" s="19"/>
+      <c r="C55" s="19"/>
+      <c r="D55" s="19"/>
+      <c r="E55" s="19"/>
+      <c r="F55" s="19"/>
+      <c r="G55" s="19"/>
+      <c r="H55" s="19"/>
+      <c r="I55" s="19"/>
+      <c r="J55" s="19"/>
+      <c r="K55" s="19"/>
+      <c r="L55" s="19"/>
+      <c r="M55" s="19"/>
+      <c r="N55" s="19"/>
+      <c r="O55" s="19"/>
+      <c r="P55" s="19"/>
+      <c r="Q55" s="19"/>
+      <c r="R55" s="19"/>
+      <c r="S55" s="19"/>
+      <c r="T55" s="19"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="16"/>
+      <c r="B56" t="s" s="23">
         <v>245</v>
       </c>
-      <c r="G53" t="s" s="23">
-        <v>75</v>
-      </c>
-      <c r="H53" t="s" s="23">
-        <v>98</v>
-      </c>
-      <c r="I53" s="24"/>
-      <c r="J53" s="24"/>
-      <c r="K53" t="s" s="23">
-        <v>58</v>
-      </c>
-      <c r="L53" t="s" s="23">
-        <v>68</v>
-      </c>
-      <c r="M53" t="s" s="23">
-        <v>99</v>
-      </c>
-      <c r="N53" s="24"/>
-      <c r="O53" t="s" s="23">
+      <c r="C56" t="s" s="23">
         <v>246</v>
       </c>
-      <c r="P53" s="24"/>
-      <c r="Q53" s="24"/>
-      <c r="R53" s="24"/>
-      <c r="S53" t="s" s="23">
-        <v>101</v>
-      </c>
-      <c r="T53" t="s" s="23">
+      <c r="D56" s="24"/>
+      <c r="E56" t="s" s="23">
+        <v>174</v>
+      </c>
+      <c r="F56" s="24"/>
+      <c r="G56" t="s" s="23">
+        <v>58</v>
+      </c>
+      <c r="H56" t="s" s="23">
+        <v>179</v>
+      </c>
+      <c r="I56" s="24"/>
+      <c r="J56" s="24"/>
+      <c r="K56" t="s" s="23">
+        <v>58</v>
+      </c>
+      <c r="L56" s="24"/>
+      <c r="M56" t="s" s="23">
         <v>247</v>
       </c>
-    </row>
-    <row r="57" s="17" customFormat="1" ht="16" customHeight="1">
-      <c r="B57" t="s" s="23">
+      <c r="N56" s="24"/>
+      <c r="O56" s="24"/>
+      <c r="P56" s="24"/>
+      <c r="Q56" s="24"/>
+      <c r="R56" s="24"/>
+      <c r="S56" t="s" s="23">
+        <v>64</v>
+      </c>
+      <c r="T56" t="s" s="23">
         <v>248</v>
       </c>
-      <c r="C57" t="s" s="23">
+    </row>
+    <row r="57" ht="13.55" customHeight="1">
+      <c r="A57" s="9"/>
+      <c r="B57" s="27"/>
+      <c r="C57" s="27"/>
+      <c r="D57" s="27"/>
+      <c r="E57" s="27"/>
+      <c r="F57" s="27"/>
+      <c r="G57" s="27"/>
+      <c r="H57" s="27"/>
+      <c r="I57" s="27"/>
+      <c r="J57" s="27"/>
+      <c r="K57" s="27"/>
+      <c r="L57" s="27"/>
+      <c r="M57" s="27"/>
+      <c r="N57" s="27"/>
+      <c r="O57" s="27"/>
+      <c r="P57" s="27"/>
+      <c r="Q57" s="27"/>
+      <c r="R57" s="27"/>
+      <c r="S57" s="27"/>
+      <c r="T57" s="27"/>
+    </row>
+    <row r="58" ht="13.55" customHeight="1">
+      <c r="A58" s="9"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+      <c r="F58" s="9"/>
+      <c r="G58" s="9"/>
+      <c r="H58" s="9"/>
+      <c r="I58" s="9"/>
+      <c r="J58" s="9"/>
+      <c r="K58" s="9"/>
+      <c r="L58" s="9"/>
+      <c r="M58" s="9"/>
+      <c r="N58" s="9"/>
+      <c r="O58" s="9"/>
+      <c r="P58" s="9"/>
+      <c r="Q58" s="9"/>
+      <c r="R58" s="9"/>
+      <c r="S58" s="9"/>
+      <c r="T58" s="9"/>
+    </row>
+    <row r="59" ht="13.55" customHeight="1">
+      <c r="A59" s="9"/>
+      <c r="B59" s="19"/>
+      <c r="C59" s="19"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
+      <c r="I59" s="9"/>
+      <c r="J59" s="9"/>
+      <c r="K59" s="9"/>
+      <c r="L59" s="9"/>
+      <c r="M59" s="9"/>
+      <c r="N59" s="9"/>
+      <c r="O59" s="9"/>
+      <c r="P59" s="9"/>
+      <c r="Q59" s="9"/>
+      <c r="R59" s="9"/>
+      <c r="S59" s="9"/>
+      <c r="T59" s="9"/>
+    </row>
+    <row r="60" ht="15" customHeight="1">
+      <c r="A60" s="16"/>
+      <c r="B60" t="s" s="20">
         <v>249</v>
       </c>
-      <c r="D57" s="24"/>
-      <c r="E57" t="s" s="23">
-        <v>174</v>
-      </c>
-      <c r="F57" s="24"/>
-      <c r="G57" t="s" s="23">
-        <v>58</v>
-      </c>
-      <c r="H57" t="s" s="23">
-        <v>179</v>
-      </c>
-      <c r="I57" s="24"/>
-      <c r="J57" s="24"/>
-      <c r="K57" t="s" s="23">
-        <v>58</v>
-      </c>
-      <c r="L57" s="24"/>
-      <c r="M57" t="s" s="23">
+      <c r="C60" s="21"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
+      <c r="G60" s="9"/>
+      <c r="H60" s="9"/>
+      <c r="I60" s="9"/>
+      <c r="J60" s="9"/>
+      <c r="K60" s="9"/>
+      <c r="L60" s="9"/>
+      <c r="M60" s="9"/>
+      <c r="N60" s="9"/>
+      <c r="O60" s="9"/>
+      <c r="P60" s="9"/>
+      <c r="Q60" s="9"/>
+      <c r="R60" s="9"/>
+      <c r="S60" s="9"/>
+      <c r="T60" s="9"/>
+    </row>
+    <row r="61" ht="15" customHeight="1">
+      <c r="A61" s="16"/>
+      <c r="B61" t="s" s="29">
         <v>250</v>
       </c>
-      <c r="N57" s="24"/>
-      <c r="O57" s="24"/>
-      <c r="P57" s="24"/>
-      <c r="Q57" s="24"/>
-      <c r="R57" s="24"/>
-      <c r="S57" t="s" s="23">
-        <v>64</v>
-      </c>
-      <c r="T57" t="s" s="23">
+      <c r="C61" s="30"/>
+      <c r="D61" s="28"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="9"/>
+      <c r="G61" s="9"/>
+      <c r="H61" s="9"/>
+      <c r="I61" s="9"/>
+      <c r="J61" s="9"/>
+      <c r="K61" s="9"/>
+      <c r="L61" s="9"/>
+      <c r="M61" s="9"/>
+      <c r="N61" s="9"/>
+      <c r="O61" s="9"/>
+      <c r="P61" s="9"/>
+      <c r="Q61" s="9"/>
+      <c r="R61" s="9"/>
+      <c r="S61" s="9"/>
+      <c r="T61" s="9"/>
+    </row>
+    <row r="62" ht="15" customHeight="1">
+      <c r="A62" s="16"/>
+      <c r="B62" t="s" s="29">
         <v>251</v>
       </c>
-    </row>
-    <row r="61" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="B61" t="s" s="20">
+      <c r="C62" s="30"/>
+      <c r="D62" s="28"/>
+      <c r="E62" s="9"/>
+      <c r="F62" s="9"/>
+      <c r="G62" s="9"/>
+      <c r="H62" s="9"/>
+      <c r="I62" s="9"/>
+      <c r="J62" s="9"/>
+      <c r="K62" s="9"/>
+      <c r="L62" s="9"/>
+      <c r="M62" s="9"/>
+      <c r="N62" s="9"/>
+      <c r="O62" s="9"/>
+      <c r="P62" s="9"/>
+      <c r="Q62" s="9"/>
+      <c r="R62" s="9"/>
+      <c r="S62" s="9"/>
+      <c r="T62" s="9"/>
+    </row>
+    <row r="63" ht="29.25" customHeight="1">
+      <c r="A63" s="16"/>
+      <c r="B63" t="s" s="31">
         <v>252</v>
       </c>
-      <c r="C61" s="21"/>
-    </row>
-    <row r="62" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="B62" t="s" s="27">
+      <c r="C63" s="32"/>
+      <c r="D63" s="28"/>
+      <c r="E63" s="9"/>
+      <c r="F63" s="9"/>
+      <c r="G63" s="9"/>
+      <c r="H63" s="9"/>
+      <c r="I63" s="9"/>
+      <c r="J63" s="9"/>
+      <c r="K63" s="9"/>
+      <c r="L63" s="9"/>
+      <c r="M63" s="9"/>
+      <c r="N63" s="9"/>
+      <c r="O63" s="9"/>
+      <c r="P63" s="9"/>
+      <c r="Q63" s="9"/>
+      <c r="R63" s="9"/>
+      <c r="S63" s="9"/>
+      <c r="T63" s="9"/>
+    </row>
+    <row r="64" ht="13.55" customHeight="1">
+      <c r="A64" s="16"/>
+      <c r="B64" t="s" s="31">
         <v>253</v>
       </c>
-      <c r="C62" s="28"/>
-    </row>
-    <row r="63" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="B63" t="s" s="27">
+      <c r="C64" s="32"/>
+      <c r="D64" s="28"/>
+      <c r="E64" s="9"/>
+      <c r="F64" s="9"/>
+      <c r="G64" s="9"/>
+      <c r="H64" s="9"/>
+      <c r="I64" s="9"/>
+      <c r="J64" s="9"/>
+      <c r="K64" s="9"/>
+      <c r="L64" s="9"/>
+      <c r="M64" s="9"/>
+      <c r="N64" s="9"/>
+      <c r="O64" s="9"/>
+      <c r="P64" s="9"/>
+      <c r="Q64" s="9"/>
+      <c r="R64" s="9"/>
+      <c r="S64" s="9"/>
+      <c r="T64" s="9"/>
+    </row>
+    <row r="65" ht="13.55" customHeight="1">
+      <c r="A65" s="16"/>
+      <c r="B65" t="s" s="31">
         <v>254</v>
       </c>
-      <c r="C63" s="28"/>
-    </row>
-    <row r="64" s="17" customFormat="1" ht="29.25" customHeight="1">
-      <c r="B64" t="s" s="29">
+      <c r="C65" s="32"/>
+      <c r="D65" s="28"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9"/>
+      <c r="G65" s="9"/>
+      <c r="H65" s="9"/>
+      <c r="I65" s="9"/>
+      <c r="J65" s="9"/>
+      <c r="K65" s="9"/>
+      <c r="L65" s="9"/>
+      <c r="M65" s="9"/>
+      <c r="N65" s="9"/>
+      <c r="O65" s="9"/>
+      <c r="P65" s="9"/>
+      <c r="Q65" s="9"/>
+      <c r="R65" s="9"/>
+      <c r="S65" s="9"/>
+      <c r="T65" s="9"/>
+    </row>
+    <row r="66" ht="13.55" customHeight="1">
+      <c r="A66" s="16"/>
+      <c r="B66" t="s" s="33">
         <v>255</v>
       </c>
-      <c r="C64" s="30"/>
-    </row>
-    <row r="65" s="17" customFormat="1" ht="13.55" customHeight="1">
-      <c r="B65" t="s" s="29">
-        <v>256</v>
-      </c>
-      <c r="C65" s="30"/>
-    </row>
-    <row r="66" s="17" customFormat="1" ht="13.55" customHeight="1">
-      <c r="B66" t="s" s="29">
-        <v>257</v>
-      </c>
-      <c r="C66" s="30"/>
-    </row>
-    <row r="67" s="17" customFormat="1" ht="13.55" customHeight="1">
-      <c r="B67" t="s" s="31">
-        <v>258</v>
-      </c>
-      <c r="C67" s="32"/>
+      <c r="C66" s="34"/>
+      <c r="D66" s="28"/>
+      <c r="E66" s="9"/>
+      <c r="F66" s="9"/>
+      <c r="G66" s="9"/>
+      <c r="H66" s="9"/>
+      <c r="I66" s="9"/>
+      <c r="J66" s="9"/>
+      <c r="K66" s="9"/>
+      <c r="L66" s="9"/>
+      <c r="M66" s="9"/>
+      <c r="N66" s="9"/>
+      <c r="O66" s="9"/>
+      <c r="P66" s="9"/>
+      <c r="Q66" s="9"/>
+      <c r="R66" s="9"/>
+      <c r="S66" s="9"/>
+      <c r="T66" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B62:C62"/>
     <mergeCell ref="B63:C63"/>
     <mergeCell ref="B64:C64"/>
     <mergeCell ref="B65:C65"/>
     <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C67"/>
     <mergeCell ref="C1:L1"/>
     <mergeCell ref="C2:L2"/>
     <mergeCell ref="C3:L3"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="C5:L5"/>
+    <mergeCell ref="B60:C60"/>
     <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
     <mergeCell ref="C6:L6"/>
     <mergeCell ref="C7:L7"/>
     <mergeCell ref="C8:L8"/>
@@ -5186,8 +5563,8 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="6" width="8.85156" style="33" customWidth="1"/>
-    <col min="7" max="16384" width="8.85156" style="33" customWidth="1"/>
+    <col min="1" max="6" width="8.85156" style="35" customWidth="1"/>
+    <col min="7" max="16384" width="8.85156" style="35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
@@ -5224,65 +5601,65 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="4"/>
-      <c r="B5" t="s" s="34">
-        <v>259</v>
-      </c>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
+      <c r="B5" t="s" s="36">
+        <v>256</v>
+      </c>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="4"/>
-      <c r="B6" t="s" s="36">
-        <v>260</v>
-      </c>
-      <c r="C6" t="s" s="37">
-        <v>261</v>
-      </c>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
+      <c r="B6" t="s" s="38">
+        <v>257</v>
+      </c>
+      <c r="C6" t="s" s="39">
+        <v>258</v>
+      </c>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="4"/>
-      <c r="B7" s="39"/>
-      <c r="C7" t="s" s="37">
-        <v>262</v>
-      </c>
-      <c r="D7" s="38"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="38"/>
+      <c r="B7" s="41"/>
+      <c r="C7" t="s" s="39">
+        <v>259</v>
+      </c>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="4"/>
-      <c r="B8" s="39"/>
-      <c r="C8" t="s" s="37">
-        <v>263</v>
-      </c>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
+      <c r="B8" s="41"/>
+      <c r="C8" t="s" s="39">
+        <v>260</v>
+      </c>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="4"/>
-      <c r="B9" s="39"/>
-      <c r="C9" t="s" s="37">
-        <v>264</v>
-      </c>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
+      <c r="B9" s="41"/>
+      <c r="C9" t="s" s="39">
+        <v>261</v>
+      </c>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="4"/>
-      <c r="B10" s="39"/>
-      <c r="C10" t="s" s="40">
-        <v>265</v>
-      </c>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="B10" s="41"/>
+      <c r="C10" t="s" s="42">
+        <v>262</v>
+      </c>
+      <c r="D10" s="43"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -5303,224 +5680,224 @@
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.85156" style="42" customWidth="1"/>
-    <col min="2" max="2" width="20.6719" style="42" customWidth="1"/>
-    <col min="3" max="3" width="16.8516" style="42" customWidth="1"/>
-    <col min="4" max="4" width="37" style="42" customWidth="1"/>
-    <col min="5" max="5" width="8.85156" style="42" customWidth="1"/>
-    <col min="6" max="16384" width="8.85156" style="42" customWidth="1"/>
+    <col min="1" max="1" width="8.85156" style="44" customWidth="1"/>
+    <col min="2" max="2" width="20.6719" style="44" customWidth="1"/>
+    <col min="3" max="3" width="16.8516" style="44" customWidth="1"/>
+    <col min="4" max="4" width="37" style="44" customWidth="1"/>
+    <col min="5" max="5" width="8.85156" style="44" customWidth="1"/>
+    <col min="6" max="16384" width="8.85156" style="44" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="2"/>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
       <c r="E1" s="2"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="44"/>
-      <c r="B2" t="s" s="45">
-        <v>266</v>
-      </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="48"/>
+      <c r="A2" s="46"/>
+      <c r="B2" t="s" s="47">
+        <v>263</v>
+      </c>
+      <c r="C2" s="48"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="50"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="44"/>
-      <c r="B3" t="s" s="49">
+      <c r="A3" s="46"/>
+      <c r="B3" t="s" s="51">
         <v>29</v>
       </c>
       <c r="C3" t="s" s="22">
         <v>31</v>
       </c>
-      <c r="D3" t="s" s="50">
+      <c r="D3" t="s" s="52">
         <v>46</v>
       </c>
-      <c r="E3" s="48"/>
+      <c r="E3" s="50"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="44"/>
-      <c r="B4" t="s" s="49">
+      <c r="A4" s="46"/>
+      <c r="B4" t="s" s="51">
         <v>2</v>
       </c>
       <c r="C4" t="s" s="22">
         <v>6</v>
       </c>
-      <c r="D4" t="s" s="50">
+      <c r="D4" t="s" s="52">
         <v>24</v>
       </c>
-      <c r="E4" s="48"/>
+      <c r="E4" s="50"/>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="4"/>
-      <c r="B5" t="s" s="51">
+      <c r="B5" t="s" s="53">
         <v>80</v>
       </c>
-      <c r="C5" t="s" s="52">
+      <c r="C5" t="s" s="54">
         <v>79</v>
       </c>
-      <c r="D5" t="s" s="53">
+      <c r="D5" t="s" s="55">
         <v>79</v>
       </c>
-      <c r="E5" s="54"/>
+      <c r="E5" s="56"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="4"/>
-      <c r="B6" t="s" s="55">
-        <v>267</v>
-      </c>
-      <c r="C6" t="s" s="56">
+      <c r="B6" t="s" s="57">
+        <v>264</v>
+      </c>
+      <c r="C6" t="s" s="58">
         <v>79</v>
       </c>
-      <c r="D6" t="s" s="57">
+      <c r="D6" t="s" s="59">
         <v>79</v>
       </c>
-      <c r="E6" s="54"/>
+      <c r="E6" s="56"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="4"/>
-      <c r="B7" t="s" s="55">
+      <c r="B7" t="s" s="57">
         <v>149</v>
       </c>
-      <c r="C7" t="s" s="56">
+      <c r="C7" t="s" s="58">
         <v>59</v>
       </c>
-      <c r="D7" t="s" s="57">
+      <c r="D7" t="s" s="59">
         <v>148</v>
       </c>
-      <c r="E7" s="54"/>
+      <c r="E7" s="56"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="4"/>
-      <c r="B8" t="s" s="55">
-        <v>244</v>
-      </c>
-      <c r="C8" t="s" s="56">
+      <c r="B8" t="s" s="57">
+        <v>241</v>
+      </c>
+      <c r="C8" t="s" s="58">
         <v>59</v>
       </c>
-      <c r="D8" t="s" s="57">
-        <v>243</v>
-      </c>
-      <c r="E8" s="54"/>
+      <c r="D8" t="s" s="59">
+        <v>240</v>
+      </c>
+      <c r="E8" s="56"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="4"/>
-      <c r="B9" t="s" s="55">
-        <v>268</v>
-      </c>
-      <c r="C9" t="s" s="56">
-        <v>269</v>
-      </c>
-      <c r="D9" t="s" s="57">
-        <v>270</v>
-      </c>
-      <c r="E9" s="54"/>
+      <c r="B9" t="s" s="57">
+        <v>265</v>
+      </c>
+      <c r="C9" t="s" s="58">
+        <v>266</v>
+      </c>
+      <c r="D9" t="s" s="59">
+        <v>267</v>
+      </c>
+      <c r="E9" s="56"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="4"/>
-      <c r="B10" t="s" s="55">
+      <c r="B10" t="s" s="57">
         <v>129</v>
       </c>
-      <c r="C10" t="s" s="56">
-        <v>271</v>
-      </c>
-      <c r="D10" t="s" s="57">
-        <v>272</v>
-      </c>
-      <c r="E10" s="54"/>
+      <c r="C10" t="s" s="58">
+        <v>268</v>
+      </c>
+      <c r="D10" t="s" s="59">
+        <v>269</v>
+      </c>
+      <c r="E10" s="56"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="4"/>
-      <c r="B11" t="s" s="55">
-        <v>273</v>
-      </c>
-      <c r="C11" t="s" s="56">
-        <v>274</v>
-      </c>
-      <c r="D11" t="s" s="57">
+      <c r="B11" t="s" s="57">
+        <v>270</v>
+      </c>
+      <c r="C11" t="s" s="58">
+        <v>271</v>
+      </c>
+      <c r="D11" t="s" s="59">
         <v>157</v>
       </c>
-      <c r="E11" s="54"/>
+      <c r="E11" s="56"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="4"/>
-      <c r="B12" t="s" s="55">
+      <c r="B12" t="s" s="57">
         <v>139</v>
       </c>
-      <c r="C12" t="s" s="56">
-        <v>275</v>
-      </c>
-      <c r="D12" t="s" s="57">
+      <c r="C12" t="s" s="58">
+        <v>272</v>
+      </c>
+      <c r="D12" t="s" s="59">
         <v>138</v>
       </c>
-      <c r="E12" s="54"/>
+      <c r="E12" s="56"/>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="4"/>
-      <c r="B13" t="s" s="55">
+      <c r="B13" t="s" s="57">
         <v>144</v>
       </c>
-      <c r="C13" t="s" s="56">
-        <v>276</v>
-      </c>
-      <c r="D13" t="s" s="57">
+      <c r="C13" t="s" s="58">
+        <v>273</v>
+      </c>
+      <c r="D13" t="s" s="59">
         <v>143</v>
       </c>
-      <c r="E13" s="54"/>
+      <c r="E13" s="56"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="4"/>
-      <c r="B14" t="s" s="55">
+      <c r="B14" t="s" s="57">
         <v>134</v>
       </c>
-      <c r="C14" t="s" s="56">
-        <v>277</v>
-      </c>
-      <c r="D14" t="s" s="57">
+      <c r="C14" t="s" s="58">
+        <v>274</v>
+      </c>
+      <c r="D14" t="s" s="59">
         <v>133</v>
       </c>
-      <c r="E14" s="54"/>
+      <c r="E14" s="56"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="4"/>
-      <c r="B15" t="s" s="55">
-        <v>278</v>
-      </c>
-      <c r="C15" t="s" s="56">
-        <v>279</v>
-      </c>
-      <c r="D15" t="s" s="57">
+      <c r="B15" t="s" s="57">
+        <v>275</v>
+      </c>
+      <c r="C15" t="s" s="58">
+        <v>276</v>
+      </c>
+      <c r="D15" t="s" s="59">
         <v>123</v>
       </c>
-      <c r="E15" s="54"/>
+      <c r="E15" s="56"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="4"/>
-      <c r="B16" t="s" s="55">
-        <v>280</v>
-      </c>
-      <c r="C16" t="s" s="56">
-        <v>281</v>
-      </c>
-      <c r="D16" t="s" s="57">
-        <v>282</v>
-      </c>
-      <c r="E16" s="54"/>
+      <c r="B16" t="s" s="57">
+        <v>277</v>
+      </c>
+      <c r="C16" t="s" s="58">
+        <v>278</v>
+      </c>
+      <c r="D16" t="s" s="59">
+        <v>279</v>
+      </c>
+      <c r="E16" s="56"/>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="4"/>
-      <c r="B17" t="s" s="58">
-        <v>283</v>
-      </c>
-      <c r="C17" t="s" s="59">
-        <v>284</v>
-      </c>
-      <c r="D17" t="s" s="60">
-        <v>285</v>
-      </c>
-      <c r="E17" s="54"/>
+      <c r="B17" t="s" s="60">
+        <v>280</v>
+      </c>
+      <c r="C17" t="s" s="61">
+        <v>281</v>
+      </c>
+      <c r="D17" t="s" s="62">
+        <v>282</v>
+      </c>
+      <c r="E17" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
EPBDS-13811 Fix trace for `origin` and `active` properties
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules/doc/TablePropertyDefinition.xlsx
+++ b/DEV/org.openl.rules/doc/TablePropertyDefinition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10410"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10512"/>
   <workbookPr autoCompressPictures="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vpikus/Sources/OpenL/openl-tablets/DEV/org.openl.rules/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF493FE-5ED0-F647-A4AE-EFCAEDF33AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE44650-3659-7344-ADC1-43A93E2F1070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="34940" windowHeight="21360" tabRatio="783" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="34940" windowHeight="21360" tabRatio="783" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Descriptions" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="291">
   <si>
     <t>Display Name</t>
   </si>
@@ -933,6 +933,9 @@
   </si>
   <si>
     <t>A Locale object represents a specific geographical, political, or cultural region.</t>
+  </si>
+  <si>
+    <t>eq(origin)</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1035,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1311,6 +1314,45 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1349,7 +1391,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1415,19 +1457,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1590,9 +1626,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1630,9 +1666,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1665,26 +1701,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1717,26 +1736,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1920,207 +1922,207 @@
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
     </row>
     <row r="3" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
     </row>
     <row r="4" spans="2:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
     </row>
     <row r="5" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
     </row>
     <row r="6" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="28"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
     </row>
     <row r="7" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="29"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" spans="2:10" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
     </row>
     <row r="9" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
     </row>
     <row r="10" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
     </row>
     <row r="11" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="28"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
     </row>
     <row r="12" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="28"/>
     </row>
     <row r="14" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="30"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28"/>
     </row>
     <row r="15" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="31"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
     </row>
@@ -2183,154 +2185,154 @@
       <c r="B1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
     </row>
     <row r="2" spans="2:20" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
     </row>
     <row r="3" spans="2:20" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="27"/>
     </row>
     <row r="4" spans="2:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="28"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
     </row>
     <row r="5" spans="2:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
     </row>
     <row r="6" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="29"/>
-      <c r="L6" s="29"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
     </row>
     <row r="7" spans="2:20" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="29"/>
-      <c r="K7" s="29"/>
-      <c r="L7" s="29"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="27"/>
     </row>
     <row r="8" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28"/>
-      <c r="K8" s="28"/>
-      <c r="L8" s="28"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
     </row>
     <row r="9" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="28"/>
-      <c r="L9" s="28"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
     </row>
     <row r="10" spans="2:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="2"/>
@@ -2342,27 +2344,27 @@
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="32"/>
-      <c r="K11" s="32"/>
-      <c r="L11" s="32"/>
-      <c r="M11" s="32"/>
-      <c r="N11" s="32"/>
-      <c r="O11" s="32"/>
-      <c r="P11" s="32"/>
-      <c r="Q11" s="32"/>
-      <c r="R11" s="32"/>
-      <c r="S11" s="32"/>
-      <c r="T11" s="32"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="30"/>
+      <c r="K11" s="30"/>
+      <c r="L11" s="30"/>
+      <c r="M11" s="30"/>
+      <c r="N11" s="30"/>
+      <c r="O11" s="30"/>
+      <c r="P11" s="30"/>
+      <c r="Q11" s="30"/>
+      <c r="R11" s="30"/>
+      <c r="S11" s="30"/>
+      <c r="T11" s="30"/>
     </row>
     <row r="12" spans="2:20" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="4" t="s">
@@ -3363,7 +3365,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="5" t="s">
         <v>216</v>
       </c>
@@ -3376,7 +3378,9 @@
       <c r="E33" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="F33" s="5"/>
+      <c r="F33" s="5" t="s">
+        <v>290</v>
+      </c>
       <c r="G33" s="5" t="s">
         <v>78</v>
       </c>
@@ -3406,7 +3410,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="34" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="5" t="s">
         <v>134</v>
       </c>
@@ -3451,7 +3455,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="35" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="5" t="s">
         <v>150</v>
       </c>
@@ -3496,7 +3500,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="36" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="5" t="s">
         <v>158</v>
       </c>
@@ -3537,7 +3541,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="37" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="5" t="s">
         <v>162</v>
       </c>
@@ -3581,7 +3585,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="38" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="5" t="s">
         <v>116</v>
       </c>
@@ -3628,7 +3632,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="39" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="5" t="s">
         <v>123</v>
       </c>
@@ -3671,7 +3675,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="5" t="s">
         <v>127</v>
       </c>
@@ -3714,7 +3718,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="41" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="5" t="s">
         <v>167</v>
       </c>
@@ -3756,7 +3760,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="42" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="5" t="s">
         <v>170</v>
       </c>
@@ -3797,8 +3801,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="43" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="25"/>
+    <row r="43" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="5" t="s">
         <v>254</v>
       </c>
@@ -3841,7 +3844,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="44" spans="1:1025" ht="32" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:20" ht="32" x14ac:dyDescent="0.2">
       <c r="B44" s="5" t="s">
         <v>175</v>
       </c>
@@ -3883,10 +3886,8 @@
       <c r="T44" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="U44" s="24"/>
-    </row>
-    <row r="45" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="24"/>
+    </row>
+    <row r="45" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="5" t="s">
         <v>248</v>
       </c>
@@ -3929,7 +3930,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="46" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B46" s="5" t="s">
         <v>181</v>
       </c>
@@ -3970,7 +3971,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="47" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="5" t="s">
         <v>183</v>
       </c>
@@ -4010,1013 +4011,8 @@
       <c r="T47" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="V47" s="23"/>
-      <c r="W47" s="23"/>
-      <c r="X47" s="23"/>
-      <c r="Y47" s="23"/>
-      <c r="Z47" s="23"/>
-      <c r="AA47" s="23"/>
-      <c r="AB47" s="23"/>
-      <c r="AC47" s="23"/>
-      <c r="AD47" s="23"/>
-      <c r="AE47" s="23"/>
-      <c r="AF47" s="23"/>
-      <c r="AG47" s="23"/>
-      <c r="AH47" s="23"/>
-      <c r="AI47" s="23"/>
-      <c r="AJ47" s="23"/>
-      <c r="AK47" s="23"/>
-      <c r="AL47" s="23"/>
-      <c r="AM47" s="23"/>
-      <c r="AN47" s="23"/>
-      <c r="AO47" s="23"/>
-      <c r="AP47" s="23"/>
-      <c r="AQ47" s="23"/>
-      <c r="AR47" s="23"/>
-      <c r="AS47" s="23"/>
-      <c r="AT47" s="23"/>
-      <c r="AU47" s="23"/>
-      <c r="AV47" s="23"/>
-      <c r="AW47" s="23"/>
-      <c r="AX47" s="23"/>
-      <c r="AY47" s="23"/>
-      <c r="AZ47" s="23"/>
-      <c r="BA47" s="23"/>
-      <c r="BB47" s="23"/>
-      <c r="BC47" s="23"/>
-      <c r="BD47" s="23"/>
-      <c r="BE47" s="23"/>
-      <c r="BF47" s="23"/>
-      <c r="BG47" s="23"/>
-      <c r="BH47" s="23"/>
-      <c r="BI47" s="23"/>
-      <c r="BJ47" s="23"/>
-      <c r="BK47" s="23"/>
-      <c r="BL47" s="23"/>
-      <c r="BM47" s="23"/>
-      <c r="BN47" s="23"/>
-      <c r="BO47" s="23"/>
-      <c r="BP47" s="23"/>
-      <c r="BQ47" s="23"/>
-      <c r="BR47" s="23"/>
-      <c r="BS47" s="23"/>
-      <c r="BT47" s="23"/>
-      <c r="BU47" s="23"/>
-      <c r="BV47" s="23"/>
-      <c r="BW47" s="23"/>
-      <c r="BX47" s="23"/>
-      <c r="BY47" s="23"/>
-      <c r="BZ47" s="23"/>
-      <c r="CA47" s="23"/>
-      <c r="CB47" s="23"/>
-      <c r="CC47" s="23"/>
-      <c r="CD47" s="23"/>
-      <c r="CE47" s="23"/>
-      <c r="CF47" s="23"/>
-      <c r="CG47" s="23"/>
-      <c r="CH47" s="23"/>
-      <c r="CI47" s="23"/>
-      <c r="CJ47" s="23"/>
-      <c r="CK47" s="23"/>
-      <c r="CL47" s="23"/>
-      <c r="CM47" s="23"/>
-      <c r="CN47" s="23"/>
-      <c r="CO47" s="23"/>
-      <c r="CP47" s="23"/>
-      <c r="CQ47" s="23"/>
-      <c r="CR47" s="23"/>
-      <c r="CS47" s="23"/>
-      <c r="CT47" s="23"/>
-      <c r="CU47" s="23"/>
-      <c r="CV47" s="23"/>
-      <c r="CW47" s="23"/>
-      <c r="CX47" s="23"/>
-      <c r="CY47" s="23"/>
-      <c r="CZ47" s="23"/>
-      <c r="DA47" s="23"/>
-      <c r="DB47" s="23"/>
-      <c r="DC47" s="23"/>
-      <c r="DD47" s="23"/>
-      <c r="DE47" s="23"/>
-      <c r="DF47" s="23"/>
-      <c r="DG47" s="23"/>
-      <c r="DH47" s="23"/>
-      <c r="DI47" s="23"/>
-      <c r="DJ47" s="23"/>
-      <c r="DK47" s="23"/>
-      <c r="DL47" s="23"/>
-      <c r="DM47" s="23"/>
-      <c r="DN47" s="23"/>
-      <c r="DO47" s="23"/>
-      <c r="DP47" s="23"/>
-      <c r="DQ47" s="23"/>
-      <c r="DR47" s="23"/>
-      <c r="DS47" s="23"/>
-      <c r="DT47" s="23"/>
-      <c r="DU47" s="23"/>
-      <c r="DV47" s="23"/>
-      <c r="DW47" s="23"/>
-      <c r="DX47" s="23"/>
-      <c r="DY47" s="23"/>
-      <c r="DZ47" s="23"/>
-      <c r="EA47" s="23"/>
-      <c r="EB47" s="23"/>
-      <c r="EC47" s="23"/>
-      <c r="ED47" s="23"/>
-      <c r="EE47" s="23"/>
-      <c r="EF47" s="23"/>
-      <c r="EG47" s="23"/>
-      <c r="EH47" s="23"/>
-      <c r="EI47" s="23"/>
-      <c r="EJ47" s="23"/>
-      <c r="EK47" s="23"/>
-      <c r="EL47" s="23"/>
-      <c r="EM47" s="23"/>
-      <c r="EN47" s="23"/>
-      <c r="EO47" s="23"/>
-      <c r="EP47" s="23"/>
-      <c r="EQ47" s="23"/>
-      <c r="ER47" s="23"/>
-      <c r="ES47" s="23"/>
-      <c r="ET47" s="23"/>
-      <c r="EU47" s="23"/>
-      <c r="EV47" s="23"/>
-      <c r="EW47" s="23"/>
-      <c r="EX47" s="23"/>
-      <c r="EY47" s="23"/>
-      <c r="EZ47" s="23"/>
-      <c r="FA47" s="23"/>
-      <c r="FB47" s="23"/>
-      <c r="FC47" s="23"/>
-      <c r="FD47" s="23"/>
-      <c r="FE47" s="23"/>
-      <c r="FF47" s="23"/>
-      <c r="FG47" s="23"/>
-      <c r="FH47" s="23"/>
-      <c r="FI47" s="23"/>
-      <c r="FJ47" s="23"/>
-      <c r="FK47" s="23"/>
-      <c r="FL47" s="23"/>
-      <c r="FM47" s="23"/>
-      <c r="FN47" s="23"/>
-      <c r="FO47" s="23"/>
-      <c r="FP47" s="23"/>
-      <c r="FQ47" s="23"/>
-      <c r="FR47" s="23"/>
-      <c r="FS47" s="23"/>
-      <c r="FT47" s="23"/>
-      <c r="FU47" s="23"/>
-      <c r="FV47" s="23"/>
-      <c r="FW47" s="23"/>
-      <c r="FX47" s="23"/>
-      <c r="FY47" s="23"/>
-      <c r="FZ47" s="23"/>
-      <c r="GA47" s="23"/>
-      <c r="GB47" s="23"/>
-      <c r="GC47" s="23"/>
-      <c r="GD47" s="23"/>
-      <c r="GE47" s="23"/>
-      <c r="GF47" s="23"/>
-      <c r="GG47" s="23"/>
-      <c r="GH47" s="23"/>
-      <c r="GI47" s="23"/>
-      <c r="GJ47" s="23"/>
-      <c r="GK47" s="23"/>
-      <c r="GL47" s="23"/>
-      <c r="GM47" s="23"/>
-      <c r="GN47" s="23"/>
-      <c r="GO47" s="23"/>
-      <c r="GP47" s="23"/>
-      <c r="GQ47" s="23"/>
-      <c r="GR47" s="23"/>
-      <c r="GS47" s="23"/>
-      <c r="GT47" s="23"/>
-      <c r="GU47" s="23"/>
-      <c r="GV47" s="23"/>
-      <c r="GW47" s="23"/>
-      <c r="GX47" s="23"/>
-      <c r="GY47" s="23"/>
-      <c r="GZ47" s="23"/>
-      <c r="HA47" s="23"/>
-      <c r="HB47" s="23"/>
-      <c r="HC47" s="23"/>
-      <c r="HD47" s="23"/>
-      <c r="HE47" s="23"/>
-      <c r="HF47" s="23"/>
-      <c r="HG47" s="23"/>
-      <c r="HH47" s="23"/>
-      <c r="HI47" s="23"/>
-      <c r="HJ47" s="23"/>
-      <c r="HK47" s="23"/>
-      <c r="HL47" s="23"/>
-      <c r="HM47" s="23"/>
-      <c r="HN47" s="23"/>
-      <c r="HO47" s="23"/>
-      <c r="HP47" s="23"/>
-      <c r="HQ47" s="23"/>
-      <c r="HR47" s="23"/>
-      <c r="HS47" s="23"/>
-      <c r="HT47" s="23"/>
-      <c r="HU47" s="23"/>
-      <c r="HV47" s="23"/>
-      <c r="HW47" s="23"/>
-      <c r="HX47" s="23"/>
-      <c r="HY47" s="23"/>
-      <c r="HZ47" s="23"/>
-      <c r="IA47" s="23"/>
-      <c r="IB47" s="23"/>
-      <c r="IC47" s="23"/>
-      <c r="ID47" s="23"/>
-      <c r="IE47" s="23"/>
-      <c r="IF47" s="23"/>
-      <c r="IG47" s="23"/>
-      <c r="IH47" s="23"/>
-      <c r="II47" s="23"/>
-      <c r="IJ47" s="23"/>
-      <c r="IK47" s="23"/>
-      <c r="IL47" s="23"/>
-      <c r="IM47" s="23"/>
-      <c r="IN47" s="23"/>
-      <c r="IO47" s="23"/>
-      <c r="IP47" s="23"/>
-      <c r="IQ47" s="23"/>
-      <c r="IR47" s="23"/>
-      <c r="IS47" s="23"/>
-      <c r="IT47" s="23"/>
-      <c r="IU47" s="23"/>
-      <c r="IV47" s="23"/>
-      <c r="IW47" s="23"/>
-      <c r="IX47" s="23"/>
-      <c r="IY47" s="23"/>
-      <c r="IZ47" s="23"/>
-      <c r="JA47" s="23"/>
-      <c r="JB47" s="23"/>
-      <c r="JC47" s="23"/>
-      <c r="JD47" s="23"/>
-      <c r="JE47" s="23"/>
-      <c r="JF47" s="23"/>
-      <c r="JG47" s="23"/>
-      <c r="JH47" s="23"/>
-      <c r="JI47" s="23"/>
-      <c r="JJ47" s="23"/>
-      <c r="JK47" s="23"/>
-      <c r="JL47" s="23"/>
-      <c r="JM47" s="23"/>
-      <c r="JN47" s="23"/>
-      <c r="JO47" s="23"/>
-      <c r="JP47" s="23"/>
-      <c r="JQ47" s="23"/>
-      <c r="JR47" s="23"/>
-      <c r="JS47" s="23"/>
-      <c r="JT47" s="23"/>
-      <c r="JU47" s="23"/>
-      <c r="JV47" s="23"/>
-      <c r="JW47" s="23"/>
-      <c r="JX47" s="23"/>
-      <c r="JY47" s="23"/>
-      <c r="JZ47" s="23"/>
-      <c r="KA47" s="23"/>
-      <c r="KB47" s="23"/>
-      <c r="KC47" s="23"/>
-      <c r="KD47" s="23"/>
-      <c r="KE47" s="23"/>
-      <c r="KF47" s="23"/>
-      <c r="KG47" s="23"/>
-      <c r="KH47" s="23"/>
-      <c r="KI47" s="23"/>
-      <c r="KJ47" s="23"/>
-      <c r="KK47" s="23"/>
-      <c r="KL47" s="23"/>
-      <c r="KM47" s="23"/>
-      <c r="KN47" s="23"/>
-      <c r="KO47" s="23"/>
-      <c r="KP47" s="23"/>
-      <c r="KQ47" s="23"/>
-      <c r="KR47" s="23"/>
-      <c r="KS47" s="23"/>
-      <c r="KT47" s="23"/>
-      <c r="KU47" s="23"/>
-      <c r="KV47" s="23"/>
-      <c r="KW47" s="23"/>
-      <c r="KX47" s="23"/>
-      <c r="KY47" s="23"/>
-      <c r="KZ47" s="23"/>
-      <c r="LA47" s="23"/>
-      <c r="LB47" s="23"/>
-      <c r="LC47" s="23"/>
-      <c r="LD47" s="23"/>
-      <c r="LE47" s="23"/>
-      <c r="LF47" s="23"/>
-      <c r="LG47" s="23"/>
-      <c r="LH47" s="23"/>
-      <c r="LI47" s="23"/>
-      <c r="LJ47" s="23"/>
-      <c r="LK47" s="23"/>
-      <c r="LL47" s="23"/>
-      <c r="LM47" s="23"/>
-      <c r="LN47" s="23"/>
-      <c r="LO47" s="23"/>
-      <c r="LP47" s="23"/>
-      <c r="LQ47" s="23"/>
-      <c r="LR47" s="23"/>
-      <c r="LS47" s="23"/>
-      <c r="LT47" s="23"/>
-      <c r="LU47" s="23"/>
-      <c r="LV47" s="23"/>
-      <c r="LW47" s="23"/>
-      <c r="LX47" s="23"/>
-      <c r="LY47" s="23"/>
-      <c r="LZ47" s="23"/>
-      <c r="MA47" s="23"/>
-      <c r="MB47" s="23"/>
-      <c r="MC47" s="23"/>
-      <c r="MD47" s="23"/>
-      <c r="ME47" s="23"/>
-      <c r="MF47" s="23"/>
-      <c r="MG47" s="23"/>
-      <c r="MH47" s="23"/>
-      <c r="MI47" s="23"/>
-      <c r="MJ47" s="23"/>
-      <c r="MK47" s="23"/>
-      <c r="ML47" s="23"/>
-      <c r="MM47" s="23"/>
-      <c r="MN47" s="23"/>
-      <c r="MO47" s="23"/>
-      <c r="MP47" s="23"/>
-      <c r="MQ47" s="23"/>
-      <c r="MR47" s="23"/>
-      <c r="MS47" s="23"/>
-      <c r="MT47" s="23"/>
-      <c r="MU47" s="23"/>
-      <c r="MV47" s="23"/>
-      <c r="MW47" s="23"/>
-      <c r="MX47" s="23"/>
-      <c r="MY47" s="23"/>
-      <c r="MZ47" s="23"/>
-      <c r="NA47" s="23"/>
-      <c r="NB47" s="23"/>
-      <c r="NC47" s="23"/>
-      <c r="ND47" s="23"/>
-      <c r="NE47" s="23"/>
-      <c r="NF47" s="23"/>
-      <c r="NG47" s="23"/>
-      <c r="NH47" s="23"/>
-      <c r="NI47" s="23"/>
-      <c r="NJ47" s="23"/>
-      <c r="NK47" s="23"/>
-      <c r="NL47" s="23"/>
-      <c r="NM47" s="23"/>
-      <c r="NN47" s="23"/>
-      <c r="NO47" s="23"/>
-      <c r="NP47" s="23"/>
-      <c r="NQ47" s="23"/>
-      <c r="NR47" s="23"/>
-      <c r="NS47" s="23"/>
-      <c r="NT47" s="23"/>
-      <c r="NU47" s="23"/>
-      <c r="NV47" s="23"/>
-      <c r="NW47" s="23"/>
-      <c r="NX47" s="23"/>
-      <c r="NY47" s="23"/>
-      <c r="NZ47" s="23"/>
-      <c r="OA47" s="23"/>
-      <c r="OB47" s="23"/>
-      <c r="OC47" s="23"/>
-      <c r="OD47" s="23"/>
-      <c r="OE47" s="23"/>
-      <c r="OF47" s="23"/>
-      <c r="OG47" s="23"/>
-      <c r="OH47" s="23"/>
-      <c r="OI47" s="23"/>
-      <c r="OJ47" s="23"/>
-      <c r="OK47" s="23"/>
-      <c r="OL47" s="23"/>
-      <c r="OM47" s="23"/>
-      <c r="ON47" s="23"/>
-      <c r="OO47" s="23"/>
-      <c r="OP47" s="23"/>
-      <c r="OQ47" s="23"/>
-      <c r="OR47" s="23"/>
-      <c r="OS47" s="23"/>
-      <c r="OT47" s="23"/>
-      <c r="OU47" s="23"/>
-      <c r="OV47" s="23"/>
-      <c r="OW47" s="23"/>
-      <c r="OX47" s="23"/>
-      <c r="OY47" s="23"/>
-      <c r="OZ47" s="23"/>
-      <c r="PA47" s="23"/>
-      <c r="PB47" s="23"/>
-      <c r="PC47" s="23"/>
-      <c r="PD47" s="23"/>
-      <c r="PE47" s="23"/>
-      <c r="PF47" s="23"/>
-      <c r="PG47" s="23"/>
-      <c r="PH47" s="23"/>
-      <c r="PI47" s="23"/>
-      <c r="PJ47" s="23"/>
-      <c r="PK47" s="23"/>
-      <c r="PL47" s="23"/>
-      <c r="PM47" s="23"/>
-      <c r="PN47" s="23"/>
-      <c r="PO47" s="23"/>
-      <c r="PP47" s="23"/>
-      <c r="PQ47" s="23"/>
-      <c r="PR47" s="23"/>
-      <c r="PS47" s="23"/>
-      <c r="PT47" s="23"/>
-      <c r="PU47" s="23"/>
-      <c r="PV47" s="23"/>
-      <c r="PW47" s="23"/>
-      <c r="PX47" s="23"/>
-      <c r="PY47" s="23"/>
-      <c r="PZ47" s="23"/>
-      <c r="QA47" s="23"/>
-      <c r="QB47" s="23"/>
-      <c r="QC47" s="23"/>
-      <c r="QD47" s="23"/>
-      <c r="QE47" s="23"/>
-      <c r="QF47" s="23"/>
-      <c r="QG47" s="23"/>
-      <c r="QH47" s="23"/>
-      <c r="QI47" s="23"/>
-      <c r="QJ47" s="23"/>
-      <c r="QK47" s="23"/>
-      <c r="QL47" s="23"/>
-      <c r="QM47" s="23"/>
-      <c r="QN47" s="23"/>
-      <c r="QO47" s="23"/>
-      <c r="QP47" s="23"/>
-      <c r="QQ47" s="23"/>
-      <c r="QR47" s="23"/>
-      <c r="QS47" s="23"/>
-      <c r="QT47" s="23"/>
-      <c r="QU47" s="23"/>
-      <c r="QV47" s="23"/>
-      <c r="QW47" s="23"/>
-      <c r="QX47" s="23"/>
-      <c r="QY47" s="23"/>
-      <c r="QZ47" s="23"/>
-      <c r="RA47" s="23"/>
-      <c r="RB47" s="23"/>
-      <c r="RC47" s="23"/>
-      <c r="RD47" s="23"/>
-      <c r="RE47" s="23"/>
-      <c r="RF47" s="23"/>
-      <c r="RG47" s="23"/>
-      <c r="RH47" s="23"/>
-      <c r="RI47" s="23"/>
-      <c r="RJ47" s="23"/>
-      <c r="RK47" s="23"/>
-      <c r="RL47" s="23"/>
-      <c r="RM47" s="23"/>
-      <c r="RN47" s="23"/>
-      <c r="RO47" s="23"/>
-      <c r="RP47" s="23"/>
-      <c r="RQ47" s="23"/>
-      <c r="RR47" s="23"/>
-      <c r="RS47" s="23"/>
-      <c r="RT47" s="23"/>
-      <c r="RU47" s="23"/>
-      <c r="RV47" s="23"/>
-      <c r="RW47" s="23"/>
-      <c r="RX47" s="23"/>
-      <c r="RY47" s="23"/>
-      <c r="RZ47" s="23"/>
-      <c r="SA47" s="23"/>
-      <c r="SB47" s="23"/>
-      <c r="SC47" s="23"/>
-      <c r="SD47" s="23"/>
-      <c r="SE47" s="23"/>
-      <c r="SF47" s="23"/>
-      <c r="SG47" s="23"/>
-      <c r="SH47" s="23"/>
-      <c r="SI47" s="23"/>
-      <c r="SJ47" s="23"/>
-      <c r="SK47" s="23"/>
-      <c r="SL47" s="23"/>
-      <c r="SM47" s="23"/>
-      <c r="SN47" s="23"/>
-      <c r="SO47" s="23"/>
-      <c r="SP47" s="23"/>
-      <c r="SQ47" s="23"/>
-      <c r="SR47" s="23"/>
-      <c r="SS47" s="23"/>
-      <c r="ST47" s="23"/>
-      <c r="SU47" s="23"/>
-      <c r="SV47" s="23"/>
-      <c r="SW47" s="23"/>
-      <c r="SX47" s="23"/>
-      <c r="SY47" s="23"/>
-      <c r="SZ47" s="23"/>
-      <c r="TA47" s="23"/>
-      <c r="TB47" s="23"/>
-      <c r="TC47" s="23"/>
-      <c r="TD47" s="23"/>
-      <c r="TE47" s="23"/>
-      <c r="TF47" s="23"/>
-      <c r="TG47" s="23"/>
-      <c r="TH47" s="23"/>
-      <c r="TI47" s="23"/>
-      <c r="TJ47" s="23"/>
-      <c r="TK47" s="23"/>
-      <c r="TL47" s="23"/>
-      <c r="TM47" s="23"/>
-      <c r="TN47" s="23"/>
-      <c r="TO47" s="23"/>
-      <c r="TP47" s="23"/>
-      <c r="TQ47" s="23"/>
-      <c r="TR47" s="23"/>
-      <c r="TS47" s="23"/>
-      <c r="TT47" s="23"/>
-      <c r="TU47" s="23"/>
-      <c r="TV47" s="23"/>
-      <c r="TW47" s="23"/>
-      <c r="TX47" s="23"/>
-      <c r="TY47" s="23"/>
-      <c r="TZ47" s="23"/>
-      <c r="UA47" s="23"/>
-      <c r="UB47" s="23"/>
-      <c r="UC47" s="23"/>
-      <c r="UD47" s="23"/>
-      <c r="UE47" s="23"/>
-      <c r="UF47" s="23"/>
-      <c r="UG47" s="23"/>
-      <c r="UH47" s="23"/>
-      <c r="UI47" s="23"/>
-      <c r="UJ47" s="23"/>
-      <c r="UK47" s="23"/>
-      <c r="UL47" s="23"/>
-      <c r="UM47" s="23"/>
-      <c r="UN47" s="23"/>
-      <c r="UO47" s="23"/>
-      <c r="UP47" s="23"/>
-      <c r="UQ47" s="23"/>
-      <c r="UR47" s="23"/>
-      <c r="US47" s="23"/>
-      <c r="UT47" s="23"/>
-      <c r="UU47" s="23"/>
-      <c r="UV47" s="23"/>
-      <c r="UW47" s="23"/>
-      <c r="UX47" s="23"/>
-      <c r="UY47" s="23"/>
-      <c r="UZ47" s="23"/>
-      <c r="VA47" s="23"/>
-      <c r="VB47" s="23"/>
-      <c r="VC47" s="23"/>
-      <c r="VD47" s="23"/>
-      <c r="VE47" s="23"/>
-      <c r="VF47" s="23"/>
-      <c r="VG47" s="23"/>
-      <c r="VH47" s="23"/>
-      <c r="VI47" s="23"/>
-      <c r="VJ47" s="23"/>
-      <c r="VK47" s="23"/>
-      <c r="VL47" s="23"/>
-      <c r="VM47" s="23"/>
-      <c r="VN47" s="23"/>
-      <c r="VO47" s="23"/>
-      <c r="VP47" s="23"/>
-      <c r="VQ47" s="23"/>
-      <c r="VR47" s="23"/>
-      <c r="VS47" s="23"/>
-      <c r="VT47" s="23"/>
-      <c r="VU47" s="23"/>
-      <c r="VV47" s="23"/>
-      <c r="VW47" s="23"/>
-      <c r="VX47" s="23"/>
-      <c r="VY47" s="23"/>
-      <c r="VZ47" s="23"/>
-      <c r="WA47" s="23"/>
-      <c r="WB47" s="23"/>
-      <c r="WC47" s="23"/>
-      <c r="WD47" s="23"/>
-      <c r="WE47" s="23"/>
-      <c r="WF47" s="23"/>
-      <c r="WG47" s="23"/>
-      <c r="WH47" s="23"/>
-      <c r="WI47" s="23"/>
-      <c r="WJ47" s="23"/>
-      <c r="WK47" s="23"/>
-      <c r="WL47" s="23"/>
-      <c r="WM47" s="23"/>
-      <c r="WN47" s="23"/>
-      <c r="WO47" s="23"/>
-      <c r="WP47" s="23"/>
-      <c r="WQ47" s="23"/>
-      <c r="WR47" s="23"/>
-      <c r="WS47" s="23"/>
-      <c r="WT47" s="23"/>
-      <c r="WU47" s="23"/>
-      <c r="WV47" s="23"/>
-      <c r="WW47" s="23"/>
-      <c r="WX47" s="23"/>
-      <c r="WY47" s="23"/>
-      <c r="WZ47" s="23"/>
-      <c r="XA47" s="23"/>
-      <c r="XB47" s="23"/>
-      <c r="XC47" s="23"/>
-      <c r="XD47" s="23"/>
-      <c r="XE47" s="23"/>
-      <c r="XF47" s="23"/>
-      <c r="XG47" s="23"/>
-      <c r="XH47" s="23"/>
-      <c r="XI47" s="23"/>
-      <c r="XJ47" s="23"/>
-      <c r="XK47" s="23"/>
-      <c r="XL47" s="23"/>
-      <c r="XM47" s="23"/>
-      <c r="XN47" s="23"/>
-      <c r="XO47" s="23"/>
-      <c r="XP47" s="23"/>
-      <c r="XQ47" s="23"/>
-      <c r="XR47" s="23"/>
-      <c r="XS47" s="23"/>
-      <c r="XT47" s="23"/>
-      <c r="XU47" s="23"/>
-      <c r="XV47" s="23"/>
-      <c r="XW47" s="23"/>
-      <c r="XX47" s="23"/>
-      <c r="XY47" s="23"/>
-      <c r="XZ47" s="23"/>
-      <c r="YA47" s="23"/>
-      <c r="YB47" s="23"/>
-      <c r="YC47" s="23"/>
-      <c r="YD47" s="23"/>
-      <c r="YE47" s="23"/>
-      <c r="YF47" s="23"/>
-      <c r="YG47" s="23"/>
-      <c r="YH47" s="23"/>
-      <c r="YI47" s="23"/>
-      <c r="YJ47" s="23"/>
-      <c r="YK47" s="23"/>
-      <c r="YL47" s="23"/>
-      <c r="YM47" s="23"/>
-      <c r="YN47" s="23"/>
-      <c r="YO47" s="23"/>
-      <c r="YP47" s="23"/>
-      <c r="YQ47" s="23"/>
-      <c r="YR47" s="23"/>
-      <c r="YS47" s="23"/>
-      <c r="YT47" s="23"/>
-      <c r="YU47" s="23"/>
-      <c r="YV47" s="23"/>
-      <c r="YW47" s="23"/>
-      <c r="YX47" s="23"/>
-      <c r="YY47" s="23"/>
-      <c r="YZ47" s="23"/>
-      <c r="ZA47" s="23"/>
-      <c r="ZB47" s="23"/>
-      <c r="ZC47" s="23"/>
-      <c r="ZD47" s="23"/>
-      <c r="ZE47" s="23"/>
-      <c r="ZF47" s="23"/>
-      <c r="ZG47" s="23"/>
-      <c r="ZH47" s="23"/>
-      <c r="ZI47" s="23"/>
-      <c r="ZJ47" s="23"/>
-      <c r="ZK47" s="23"/>
-      <c r="ZL47" s="23"/>
-      <c r="ZM47" s="23"/>
-      <c r="ZN47" s="23"/>
-      <c r="ZO47" s="23"/>
-      <c r="ZP47" s="23"/>
-      <c r="ZQ47" s="23"/>
-      <c r="ZR47" s="23"/>
-      <c r="ZS47" s="23"/>
-      <c r="ZT47" s="23"/>
-      <c r="ZU47" s="23"/>
-      <c r="ZV47" s="23"/>
-      <c r="ZW47" s="23"/>
-      <c r="ZX47" s="23"/>
-      <c r="ZY47" s="23"/>
-      <c r="ZZ47" s="23"/>
-      <c r="AAA47" s="23"/>
-      <c r="AAB47" s="23"/>
-      <c r="AAC47" s="23"/>
-      <c r="AAD47" s="23"/>
-      <c r="AAE47" s="23"/>
-      <c r="AAF47" s="23"/>
-      <c r="AAG47" s="23"/>
-      <c r="AAH47" s="23"/>
-      <c r="AAI47" s="23"/>
-      <c r="AAJ47" s="23"/>
-      <c r="AAK47" s="23"/>
-      <c r="AAL47" s="23"/>
-      <c r="AAM47" s="23"/>
-      <c r="AAN47" s="23"/>
-      <c r="AAO47" s="23"/>
-      <c r="AAP47" s="23"/>
-      <c r="AAQ47" s="23"/>
-      <c r="AAR47" s="23"/>
-      <c r="AAS47" s="23"/>
-      <c r="AAT47" s="23"/>
-      <c r="AAU47" s="23"/>
-      <c r="AAV47" s="23"/>
-      <c r="AAW47" s="23"/>
-      <c r="AAX47" s="23"/>
-      <c r="AAY47" s="23"/>
-      <c r="AAZ47" s="23"/>
-      <c r="ABA47" s="23"/>
-      <c r="ABB47" s="23"/>
-      <c r="ABC47" s="23"/>
-      <c r="ABD47" s="23"/>
-      <c r="ABE47" s="23"/>
-      <c r="ABF47" s="23"/>
-      <c r="ABG47" s="23"/>
-      <c r="ABH47" s="23"/>
-      <c r="ABI47" s="23"/>
-      <c r="ABJ47" s="23"/>
-      <c r="ABK47" s="23"/>
-      <c r="ABL47" s="23"/>
-      <c r="ABM47" s="23"/>
-      <c r="ABN47" s="23"/>
-      <c r="ABO47" s="23"/>
-      <c r="ABP47" s="23"/>
-      <c r="ABQ47" s="23"/>
-      <c r="ABR47" s="23"/>
-      <c r="ABS47" s="23"/>
-      <c r="ABT47" s="23"/>
-      <c r="ABU47" s="23"/>
-      <c r="ABV47" s="23"/>
-      <c r="ABW47" s="23"/>
-      <c r="ABX47" s="23"/>
-      <c r="ABY47" s="23"/>
-      <c r="ABZ47" s="23"/>
-      <c r="ACA47" s="23"/>
-      <c r="ACB47" s="23"/>
-      <c r="ACC47" s="23"/>
-      <c r="ACD47" s="23"/>
-      <c r="ACE47" s="23"/>
-      <c r="ACF47" s="23"/>
-      <c r="ACG47" s="23"/>
-      <c r="ACH47" s="23"/>
-      <c r="ACI47" s="23"/>
-      <c r="ACJ47" s="23"/>
-      <c r="ACK47" s="23"/>
-      <c r="ACL47" s="23"/>
-      <c r="ACM47" s="23"/>
-      <c r="ACN47" s="23"/>
-      <c r="ACO47" s="23"/>
-      <c r="ACP47" s="23"/>
-      <c r="ACQ47" s="23"/>
-      <c r="ACR47" s="23"/>
-      <c r="ACS47" s="23"/>
-      <c r="ACT47" s="23"/>
-      <c r="ACU47" s="23"/>
-      <c r="ACV47" s="23"/>
-      <c r="ACW47" s="23"/>
-      <c r="ACX47" s="23"/>
-      <c r="ACY47" s="23"/>
-      <c r="ACZ47" s="23"/>
-      <c r="ADA47" s="23"/>
-      <c r="ADB47" s="23"/>
-      <c r="ADC47" s="23"/>
-      <c r="ADD47" s="23"/>
-      <c r="ADE47" s="23"/>
-      <c r="ADF47" s="23"/>
-      <c r="ADG47" s="23"/>
-      <c r="ADH47" s="23"/>
-      <c r="ADI47" s="23"/>
-      <c r="ADJ47" s="23"/>
-      <c r="ADK47" s="23"/>
-      <c r="ADL47" s="23"/>
-      <c r="ADM47" s="23"/>
-      <c r="ADN47" s="23"/>
-      <c r="ADO47" s="23"/>
-      <c r="ADP47" s="23"/>
-      <c r="ADQ47" s="23"/>
-      <c r="ADR47" s="23"/>
-      <c r="ADS47" s="23"/>
-      <c r="ADT47" s="23"/>
-      <c r="ADU47" s="23"/>
-      <c r="ADV47" s="23"/>
-      <c r="ADW47" s="23"/>
-      <c r="ADX47" s="23"/>
-      <c r="ADY47" s="23"/>
-      <c r="ADZ47" s="23"/>
-      <c r="AEA47" s="23"/>
-      <c r="AEB47" s="23"/>
-      <c r="AEC47" s="23"/>
-      <c r="AED47" s="23"/>
-      <c r="AEE47" s="23"/>
-      <c r="AEF47" s="23"/>
-      <c r="AEG47" s="23"/>
-      <c r="AEH47" s="23"/>
-      <c r="AEI47" s="23"/>
-      <c r="AEJ47" s="23"/>
-      <c r="AEK47" s="23"/>
-      <c r="AEL47" s="23"/>
-      <c r="AEM47" s="23"/>
-      <c r="AEN47" s="23"/>
-      <c r="AEO47" s="23"/>
-      <c r="AEP47" s="23"/>
-      <c r="AEQ47" s="23"/>
-      <c r="AER47" s="23"/>
-      <c r="AES47" s="23"/>
-      <c r="AET47" s="23"/>
-      <c r="AEU47" s="23"/>
-      <c r="AEV47" s="23"/>
-      <c r="AEW47" s="23"/>
-      <c r="AEX47" s="23"/>
-      <c r="AEY47" s="23"/>
-      <c r="AEZ47" s="23"/>
-      <c r="AFA47" s="23"/>
-      <c r="AFB47" s="23"/>
-      <c r="AFC47" s="23"/>
-      <c r="AFD47" s="23"/>
-      <c r="AFE47" s="23"/>
-      <c r="AFF47" s="23"/>
-      <c r="AFG47" s="23"/>
-      <c r="AFH47" s="23"/>
-      <c r="AFI47" s="23"/>
-      <c r="AFJ47" s="23"/>
-      <c r="AFK47" s="23"/>
-      <c r="AFL47" s="23"/>
-      <c r="AFM47" s="23"/>
-      <c r="AFN47" s="23"/>
-      <c r="AFO47" s="23"/>
-      <c r="AFP47" s="23"/>
-      <c r="AFQ47" s="23"/>
-      <c r="AFR47" s="23"/>
-      <c r="AFS47" s="23"/>
-      <c r="AFT47" s="23"/>
-      <c r="AFU47" s="23"/>
-      <c r="AFV47" s="23"/>
-      <c r="AFW47" s="23"/>
-      <c r="AFX47" s="23"/>
-      <c r="AFY47" s="23"/>
-      <c r="AFZ47" s="23"/>
-      <c r="AGA47" s="23"/>
-      <c r="AGB47" s="23"/>
-      <c r="AGC47" s="23"/>
-      <c r="AGD47" s="23"/>
-      <c r="AGE47" s="23"/>
-      <c r="AGF47" s="23"/>
-      <c r="AGG47" s="23"/>
-      <c r="AGH47" s="23"/>
-      <c r="AGI47" s="23"/>
-      <c r="AGJ47" s="23"/>
-      <c r="AGK47" s="23"/>
-      <c r="AGL47" s="23"/>
-      <c r="AGM47" s="23"/>
-      <c r="AGN47" s="23"/>
-      <c r="AGO47" s="23"/>
-      <c r="AGP47" s="23"/>
-      <c r="AGQ47" s="23"/>
-      <c r="AGR47" s="23"/>
-      <c r="AGS47" s="23"/>
-      <c r="AGT47" s="23"/>
-      <c r="AGU47" s="23"/>
-      <c r="AGV47" s="23"/>
-      <c r="AGW47" s="23"/>
-      <c r="AGX47" s="23"/>
-      <c r="AGY47" s="23"/>
-      <c r="AGZ47" s="23"/>
-      <c r="AHA47" s="23"/>
-      <c r="AHB47" s="23"/>
-      <c r="AHC47" s="23"/>
-      <c r="AHD47" s="23"/>
-      <c r="AHE47" s="23"/>
-      <c r="AHF47" s="23"/>
-      <c r="AHG47" s="23"/>
-      <c r="AHH47" s="23"/>
-      <c r="AHI47" s="23"/>
-      <c r="AHJ47" s="23"/>
-      <c r="AHK47" s="23"/>
-      <c r="AHL47" s="23"/>
-      <c r="AHM47" s="23"/>
-      <c r="AHN47" s="23"/>
-      <c r="AHO47" s="23"/>
-      <c r="AHP47" s="23"/>
-      <c r="AHQ47" s="23"/>
-      <c r="AHR47" s="23"/>
-      <c r="AHS47" s="23"/>
-      <c r="AHT47" s="23"/>
-      <c r="AHU47" s="23"/>
-      <c r="AHV47" s="23"/>
-      <c r="AHW47" s="23"/>
-      <c r="AHX47" s="23"/>
-      <c r="AHY47" s="23"/>
-      <c r="AHZ47" s="23"/>
-      <c r="AIA47" s="23"/>
-      <c r="AIB47" s="23"/>
-      <c r="AIC47" s="23"/>
-      <c r="AID47" s="23"/>
-      <c r="AIE47" s="23"/>
-      <c r="AIF47" s="23"/>
-      <c r="AIG47" s="23"/>
-      <c r="AIH47" s="23"/>
-      <c r="AII47" s="23"/>
-      <c r="AIJ47" s="23"/>
-      <c r="AIK47" s="23"/>
-      <c r="AIL47" s="23"/>
-      <c r="AIM47" s="23"/>
-      <c r="AIN47" s="23"/>
-      <c r="AIO47" s="23"/>
-      <c r="AIP47" s="23"/>
-      <c r="AIQ47" s="23"/>
-      <c r="AIR47" s="23"/>
-      <c r="AIS47" s="23"/>
-      <c r="AIT47" s="23"/>
-      <c r="AIU47" s="23"/>
-      <c r="AIV47" s="23"/>
-      <c r="AIW47" s="23"/>
-      <c r="AIX47" s="23"/>
-      <c r="AIY47" s="23"/>
-      <c r="AIZ47" s="23"/>
-      <c r="AJA47" s="23"/>
-      <c r="AJB47" s="23"/>
-      <c r="AJC47" s="23"/>
-      <c r="AJD47" s="23"/>
-      <c r="AJE47" s="23"/>
-      <c r="AJF47" s="23"/>
-      <c r="AJG47" s="23"/>
-      <c r="AJH47" s="23"/>
-      <c r="AJI47" s="23"/>
-      <c r="AJJ47" s="23"/>
-      <c r="AJK47" s="23"/>
-      <c r="AJL47" s="23"/>
-      <c r="AJM47" s="23"/>
-      <c r="AJN47" s="23"/>
-      <c r="AJO47" s="23"/>
-      <c r="AJP47" s="23"/>
-      <c r="AJQ47" s="23"/>
-      <c r="AJR47" s="23"/>
-      <c r="AJS47" s="23"/>
-      <c r="AJT47" s="23"/>
-      <c r="AJU47" s="23"/>
-      <c r="AJV47" s="23"/>
-      <c r="AJW47" s="23"/>
-      <c r="AJX47" s="23"/>
-      <c r="AJY47" s="23"/>
-      <c r="AJZ47" s="23"/>
-      <c r="AKA47" s="23"/>
-      <c r="AKB47" s="23"/>
-      <c r="AKC47" s="23"/>
-      <c r="AKD47" s="23"/>
-      <c r="AKE47" s="23"/>
-      <c r="AKF47" s="23"/>
-      <c r="AKG47" s="23"/>
-      <c r="AKH47" s="23"/>
-      <c r="AKI47" s="23"/>
-      <c r="AKJ47" s="23"/>
-      <c r="AKK47" s="23"/>
-      <c r="AKL47" s="23"/>
-      <c r="AKM47" s="23"/>
-      <c r="AKN47" s="23"/>
-      <c r="AKO47" s="23"/>
-      <c r="AKP47" s="23"/>
-      <c r="AKQ47" s="23"/>
-      <c r="AKR47" s="23"/>
-      <c r="AKS47" s="23"/>
-      <c r="AKT47" s="23"/>
-      <c r="AKU47" s="23"/>
-      <c r="AKV47" s="23"/>
-      <c r="AKW47" s="23"/>
-      <c r="AKX47" s="23"/>
-      <c r="AKY47" s="23"/>
-      <c r="AKZ47" s="23"/>
-      <c r="ALA47" s="23"/>
-      <c r="ALB47" s="23"/>
-      <c r="ALC47" s="23"/>
-      <c r="ALD47" s="23"/>
-      <c r="ALE47" s="23"/>
-      <c r="ALF47" s="23"/>
-      <c r="ALG47" s="23"/>
-      <c r="ALH47" s="23"/>
-      <c r="ALI47" s="23"/>
-      <c r="ALJ47" s="23"/>
-      <c r="ALK47" s="23"/>
-      <c r="ALL47" s="23"/>
-      <c r="ALM47" s="23"/>
-      <c r="ALN47" s="23"/>
-      <c r="ALO47" s="23"/>
-      <c r="ALP47" s="23"/>
-      <c r="ALQ47" s="23"/>
-      <c r="ALR47" s="23"/>
-      <c r="ALS47" s="23"/>
-      <c r="ALT47" s="23"/>
-      <c r="ALU47" s="23"/>
-      <c r="ALV47" s="23"/>
-      <c r="ALW47" s="23"/>
-      <c r="ALX47" s="23"/>
-      <c r="ALY47" s="23"/>
-      <c r="ALZ47" s="23"/>
-      <c r="AMA47" s="23"/>
-      <c r="AMB47" s="23"/>
-      <c r="AMC47" s="23"/>
-      <c r="AMD47" s="23"/>
-      <c r="AME47" s="23"/>
-      <c r="AMF47" s="23"/>
-      <c r="AMG47" s="23"/>
-      <c r="AMH47" s="23"/>
-      <c r="AMI47" s="23"/>
-      <c r="AMJ47" s="23"/>
-      <c r="AMK47" s="23"/>
-    </row>
-    <row r="48" spans="1:1025" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="27"/>
+    </row>
+    <row r="48" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="5" t="s">
         <v>282</v>
       </c>
@@ -5058,1013 +4054,8 @@
       <c r="T48" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="U48" s="27"/>
-      <c r="V48" s="27"/>
-      <c r="W48" s="27"/>
-      <c r="X48" s="27"/>
-      <c r="Y48" s="27"/>
-      <c r="Z48" s="27"/>
-      <c r="AA48" s="27"/>
-      <c r="AB48" s="27"/>
-      <c r="AC48" s="27"/>
-      <c r="AD48" s="27"/>
-      <c r="AE48" s="27"/>
-      <c r="AF48" s="27"/>
-      <c r="AG48" s="27"/>
-      <c r="AH48" s="27"/>
-      <c r="AI48" s="27"/>
-      <c r="AJ48" s="27"/>
-      <c r="AK48" s="27"/>
-      <c r="AL48" s="27"/>
-      <c r="AM48" s="27"/>
-      <c r="AN48" s="27"/>
-      <c r="AO48" s="27"/>
-      <c r="AP48" s="27"/>
-      <c r="AQ48" s="27"/>
-      <c r="AR48" s="27"/>
-      <c r="AS48" s="27"/>
-      <c r="AT48" s="27"/>
-      <c r="AU48" s="27"/>
-      <c r="AV48" s="27"/>
-      <c r="AW48" s="27"/>
-      <c r="AX48" s="27"/>
-      <c r="AY48" s="27"/>
-      <c r="AZ48" s="27"/>
-      <c r="BA48" s="27"/>
-      <c r="BB48" s="27"/>
-      <c r="BC48" s="27"/>
-      <c r="BD48" s="27"/>
-      <c r="BE48" s="27"/>
-      <c r="BF48" s="27"/>
-      <c r="BG48" s="27"/>
-      <c r="BH48" s="27"/>
-      <c r="BI48" s="27"/>
-      <c r="BJ48" s="27"/>
-      <c r="BK48" s="27"/>
-      <c r="BL48" s="27"/>
-      <c r="BM48" s="27"/>
-      <c r="BN48" s="27"/>
-      <c r="BO48" s="27"/>
-      <c r="BP48" s="27"/>
-      <c r="BQ48" s="27"/>
-      <c r="BR48" s="27"/>
-      <c r="BS48" s="27"/>
-      <c r="BT48" s="27"/>
-      <c r="BU48" s="27"/>
-      <c r="BV48" s="27"/>
-      <c r="BW48" s="27"/>
-      <c r="BX48" s="27"/>
-      <c r="BY48" s="27"/>
-      <c r="BZ48" s="27"/>
-      <c r="CA48" s="27"/>
-      <c r="CB48" s="27"/>
-      <c r="CC48" s="27"/>
-      <c r="CD48" s="27"/>
-      <c r="CE48" s="27"/>
-      <c r="CF48" s="27"/>
-      <c r="CG48" s="27"/>
-      <c r="CH48" s="27"/>
-      <c r="CI48" s="27"/>
-      <c r="CJ48" s="27"/>
-      <c r="CK48" s="27"/>
-      <c r="CL48" s="27"/>
-      <c r="CM48" s="27"/>
-      <c r="CN48" s="27"/>
-      <c r="CO48" s="27"/>
-      <c r="CP48" s="27"/>
-      <c r="CQ48" s="27"/>
-      <c r="CR48" s="27"/>
-      <c r="CS48" s="27"/>
-      <c r="CT48" s="27"/>
-      <c r="CU48" s="27"/>
-      <c r="CV48" s="27"/>
-      <c r="CW48" s="27"/>
-      <c r="CX48" s="27"/>
-      <c r="CY48" s="27"/>
-      <c r="CZ48" s="27"/>
-      <c r="DA48" s="27"/>
-      <c r="DB48" s="27"/>
-      <c r="DC48" s="27"/>
-      <c r="DD48" s="27"/>
-      <c r="DE48" s="27"/>
-      <c r="DF48" s="27"/>
-      <c r="DG48" s="27"/>
-      <c r="DH48" s="27"/>
-      <c r="DI48" s="27"/>
-      <c r="DJ48" s="27"/>
-      <c r="DK48" s="27"/>
-      <c r="DL48" s="27"/>
-      <c r="DM48" s="27"/>
-      <c r="DN48" s="27"/>
-      <c r="DO48" s="27"/>
-      <c r="DP48" s="27"/>
-      <c r="DQ48" s="27"/>
-      <c r="DR48" s="27"/>
-      <c r="DS48" s="27"/>
-      <c r="DT48" s="27"/>
-      <c r="DU48" s="27"/>
-      <c r="DV48" s="27"/>
-      <c r="DW48" s="27"/>
-      <c r="DX48" s="27"/>
-      <c r="DY48" s="27"/>
-      <c r="DZ48" s="27"/>
-      <c r="EA48" s="27"/>
-      <c r="EB48" s="27"/>
-      <c r="EC48" s="27"/>
-      <c r="ED48" s="27"/>
-      <c r="EE48" s="27"/>
-      <c r="EF48" s="27"/>
-      <c r="EG48" s="27"/>
-      <c r="EH48" s="27"/>
-      <c r="EI48" s="27"/>
-      <c r="EJ48" s="27"/>
-      <c r="EK48" s="27"/>
-      <c r="EL48" s="27"/>
-      <c r="EM48" s="27"/>
-      <c r="EN48" s="27"/>
-      <c r="EO48" s="27"/>
-      <c r="EP48" s="27"/>
-      <c r="EQ48" s="27"/>
-      <c r="ER48" s="27"/>
-      <c r="ES48" s="27"/>
-      <c r="ET48" s="27"/>
-      <c r="EU48" s="27"/>
-      <c r="EV48" s="27"/>
-      <c r="EW48" s="27"/>
-      <c r="EX48" s="27"/>
-      <c r="EY48" s="27"/>
-      <c r="EZ48" s="27"/>
-      <c r="FA48" s="27"/>
-      <c r="FB48" s="27"/>
-      <c r="FC48" s="27"/>
-      <c r="FD48" s="27"/>
-      <c r="FE48" s="27"/>
-      <c r="FF48" s="27"/>
-      <c r="FG48" s="27"/>
-      <c r="FH48" s="27"/>
-      <c r="FI48" s="27"/>
-      <c r="FJ48" s="27"/>
-      <c r="FK48" s="27"/>
-      <c r="FL48" s="27"/>
-      <c r="FM48" s="27"/>
-      <c r="FN48" s="27"/>
-      <c r="FO48" s="27"/>
-      <c r="FP48" s="27"/>
-      <c r="FQ48" s="27"/>
-      <c r="FR48" s="27"/>
-      <c r="FS48" s="27"/>
-      <c r="FT48" s="27"/>
-      <c r="FU48" s="27"/>
-      <c r="FV48" s="27"/>
-      <c r="FW48" s="27"/>
-      <c r="FX48" s="27"/>
-      <c r="FY48" s="27"/>
-      <c r="FZ48" s="27"/>
-      <c r="GA48" s="27"/>
-      <c r="GB48" s="27"/>
-      <c r="GC48" s="27"/>
-      <c r="GD48" s="27"/>
-      <c r="GE48" s="27"/>
-      <c r="GF48" s="27"/>
-      <c r="GG48" s="27"/>
-      <c r="GH48" s="27"/>
-      <c r="GI48" s="27"/>
-      <c r="GJ48" s="27"/>
-      <c r="GK48" s="27"/>
-      <c r="GL48" s="27"/>
-      <c r="GM48" s="27"/>
-      <c r="GN48" s="27"/>
-      <c r="GO48" s="27"/>
-      <c r="GP48" s="27"/>
-      <c r="GQ48" s="27"/>
-      <c r="GR48" s="27"/>
-      <c r="GS48" s="27"/>
-      <c r="GT48" s="27"/>
-      <c r="GU48" s="27"/>
-      <c r="GV48" s="27"/>
-      <c r="GW48" s="27"/>
-      <c r="GX48" s="27"/>
-      <c r="GY48" s="27"/>
-      <c r="GZ48" s="27"/>
-      <c r="HA48" s="27"/>
-      <c r="HB48" s="27"/>
-      <c r="HC48" s="27"/>
-      <c r="HD48" s="27"/>
-      <c r="HE48" s="27"/>
-      <c r="HF48" s="27"/>
-      <c r="HG48" s="27"/>
-      <c r="HH48" s="27"/>
-      <c r="HI48" s="27"/>
-      <c r="HJ48" s="27"/>
-      <c r="HK48" s="27"/>
-      <c r="HL48" s="27"/>
-      <c r="HM48" s="27"/>
-      <c r="HN48" s="27"/>
-      <c r="HO48" s="27"/>
-      <c r="HP48" s="27"/>
-      <c r="HQ48" s="27"/>
-      <c r="HR48" s="27"/>
-      <c r="HS48" s="27"/>
-      <c r="HT48" s="27"/>
-      <c r="HU48" s="27"/>
-      <c r="HV48" s="27"/>
-      <c r="HW48" s="27"/>
-      <c r="HX48" s="27"/>
-      <c r="HY48" s="27"/>
-      <c r="HZ48" s="27"/>
-      <c r="IA48" s="27"/>
-      <c r="IB48" s="27"/>
-      <c r="IC48" s="27"/>
-      <c r="ID48" s="27"/>
-      <c r="IE48" s="27"/>
-      <c r="IF48" s="27"/>
-      <c r="IG48" s="27"/>
-      <c r="IH48" s="27"/>
-      <c r="II48" s="27"/>
-      <c r="IJ48" s="27"/>
-      <c r="IK48" s="27"/>
-      <c r="IL48" s="27"/>
-      <c r="IM48" s="27"/>
-      <c r="IN48" s="27"/>
-      <c r="IO48" s="27"/>
-      <c r="IP48" s="27"/>
-      <c r="IQ48" s="27"/>
-      <c r="IR48" s="27"/>
-      <c r="IS48" s="27"/>
-      <c r="IT48" s="27"/>
-      <c r="IU48" s="27"/>
-      <c r="IV48" s="27"/>
-      <c r="IW48" s="27"/>
-      <c r="IX48" s="27"/>
-      <c r="IY48" s="27"/>
-      <c r="IZ48" s="27"/>
-      <c r="JA48" s="27"/>
-      <c r="JB48" s="27"/>
-      <c r="JC48" s="27"/>
-      <c r="JD48" s="27"/>
-      <c r="JE48" s="27"/>
-      <c r="JF48" s="27"/>
-      <c r="JG48" s="27"/>
-      <c r="JH48" s="27"/>
-      <c r="JI48" s="27"/>
-      <c r="JJ48" s="27"/>
-      <c r="JK48" s="27"/>
-      <c r="JL48" s="27"/>
-      <c r="JM48" s="27"/>
-      <c r="JN48" s="27"/>
-      <c r="JO48" s="27"/>
-      <c r="JP48" s="27"/>
-      <c r="JQ48" s="27"/>
-      <c r="JR48" s="27"/>
-      <c r="JS48" s="27"/>
-      <c r="JT48" s="27"/>
-      <c r="JU48" s="27"/>
-      <c r="JV48" s="27"/>
-      <c r="JW48" s="27"/>
-      <c r="JX48" s="27"/>
-      <c r="JY48" s="27"/>
-      <c r="JZ48" s="27"/>
-      <c r="KA48" s="27"/>
-      <c r="KB48" s="27"/>
-      <c r="KC48" s="27"/>
-      <c r="KD48" s="27"/>
-      <c r="KE48" s="27"/>
-      <c r="KF48" s="27"/>
-      <c r="KG48" s="27"/>
-      <c r="KH48" s="27"/>
-      <c r="KI48" s="27"/>
-      <c r="KJ48" s="27"/>
-      <c r="KK48" s="27"/>
-      <c r="KL48" s="27"/>
-      <c r="KM48" s="27"/>
-      <c r="KN48" s="27"/>
-      <c r="KO48" s="27"/>
-      <c r="KP48" s="27"/>
-      <c r="KQ48" s="27"/>
-      <c r="KR48" s="27"/>
-      <c r="KS48" s="27"/>
-      <c r="KT48" s="27"/>
-      <c r="KU48" s="27"/>
-      <c r="KV48" s="27"/>
-      <c r="KW48" s="27"/>
-      <c r="KX48" s="27"/>
-      <c r="KY48" s="27"/>
-      <c r="KZ48" s="27"/>
-      <c r="LA48" s="27"/>
-      <c r="LB48" s="27"/>
-      <c r="LC48" s="27"/>
-      <c r="LD48" s="27"/>
-      <c r="LE48" s="27"/>
-      <c r="LF48" s="27"/>
-      <c r="LG48" s="27"/>
-      <c r="LH48" s="27"/>
-      <c r="LI48" s="27"/>
-      <c r="LJ48" s="27"/>
-      <c r="LK48" s="27"/>
-      <c r="LL48" s="27"/>
-      <c r="LM48" s="27"/>
-      <c r="LN48" s="27"/>
-      <c r="LO48" s="27"/>
-      <c r="LP48" s="27"/>
-      <c r="LQ48" s="27"/>
-      <c r="LR48" s="27"/>
-      <c r="LS48" s="27"/>
-      <c r="LT48" s="27"/>
-      <c r="LU48" s="27"/>
-      <c r="LV48" s="27"/>
-      <c r="LW48" s="27"/>
-      <c r="LX48" s="27"/>
-      <c r="LY48" s="27"/>
-      <c r="LZ48" s="27"/>
-      <c r="MA48" s="27"/>
-      <c r="MB48" s="27"/>
-      <c r="MC48" s="27"/>
-      <c r="MD48" s="27"/>
-      <c r="ME48" s="27"/>
-      <c r="MF48" s="27"/>
-      <c r="MG48" s="27"/>
-      <c r="MH48" s="27"/>
-      <c r="MI48" s="27"/>
-      <c r="MJ48" s="27"/>
-      <c r="MK48" s="27"/>
-      <c r="ML48" s="27"/>
-      <c r="MM48" s="27"/>
-      <c r="MN48" s="27"/>
-      <c r="MO48" s="27"/>
-      <c r="MP48" s="27"/>
-      <c r="MQ48" s="27"/>
-      <c r="MR48" s="27"/>
-      <c r="MS48" s="27"/>
-      <c r="MT48" s="27"/>
-      <c r="MU48" s="27"/>
-      <c r="MV48" s="27"/>
-      <c r="MW48" s="27"/>
-      <c r="MX48" s="27"/>
-      <c r="MY48" s="27"/>
-      <c r="MZ48" s="27"/>
-      <c r="NA48" s="27"/>
-      <c r="NB48" s="27"/>
-      <c r="NC48" s="27"/>
-      <c r="ND48" s="27"/>
-      <c r="NE48" s="27"/>
-      <c r="NF48" s="27"/>
-      <c r="NG48" s="27"/>
-      <c r="NH48" s="27"/>
-      <c r="NI48" s="27"/>
-      <c r="NJ48" s="27"/>
-      <c r="NK48" s="27"/>
-      <c r="NL48" s="27"/>
-      <c r="NM48" s="27"/>
-      <c r="NN48" s="27"/>
-      <c r="NO48" s="27"/>
-      <c r="NP48" s="27"/>
-      <c r="NQ48" s="27"/>
-      <c r="NR48" s="27"/>
-      <c r="NS48" s="27"/>
-      <c r="NT48" s="27"/>
-      <c r="NU48" s="27"/>
-      <c r="NV48" s="27"/>
-      <c r="NW48" s="27"/>
-      <c r="NX48" s="27"/>
-      <c r="NY48" s="27"/>
-      <c r="NZ48" s="27"/>
-      <c r="OA48" s="27"/>
-      <c r="OB48" s="27"/>
-      <c r="OC48" s="27"/>
-      <c r="OD48" s="27"/>
-      <c r="OE48" s="27"/>
-      <c r="OF48" s="27"/>
-      <c r="OG48" s="27"/>
-      <c r="OH48" s="27"/>
-      <c r="OI48" s="27"/>
-      <c r="OJ48" s="27"/>
-      <c r="OK48" s="27"/>
-      <c r="OL48" s="27"/>
-      <c r="OM48" s="27"/>
-      <c r="ON48" s="27"/>
-      <c r="OO48" s="27"/>
-      <c r="OP48" s="27"/>
-      <c r="OQ48" s="27"/>
-      <c r="OR48" s="27"/>
-      <c r="OS48" s="27"/>
-      <c r="OT48" s="27"/>
-      <c r="OU48" s="27"/>
-      <c r="OV48" s="27"/>
-      <c r="OW48" s="27"/>
-      <c r="OX48" s="27"/>
-      <c r="OY48" s="27"/>
-      <c r="OZ48" s="27"/>
-      <c r="PA48" s="27"/>
-      <c r="PB48" s="27"/>
-      <c r="PC48" s="27"/>
-      <c r="PD48" s="27"/>
-      <c r="PE48" s="27"/>
-      <c r="PF48" s="27"/>
-      <c r="PG48" s="27"/>
-      <c r="PH48" s="27"/>
-      <c r="PI48" s="27"/>
-      <c r="PJ48" s="27"/>
-      <c r="PK48" s="27"/>
-      <c r="PL48" s="27"/>
-      <c r="PM48" s="27"/>
-      <c r="PN48" s="27"/>
-      <c r="PO48" s="27"/>
-      <c r="PP48" s="27"/>
-      <c r="PQ48" s="27"/>
-      <c r="PR48" s="27"/>
-      <c r="PS48" s="27"/>
-      <c r="PT48" s="27"/>
-      <c r="PU48" s="27"/>
-      <c r="PV48" s="27"/>
-      <c r="PW48" s="27"/>
-      <c r="PX48" s="27"/>
-      <c r="PY48" s="27"/>
-      <c r="PZ48" s="27"/>
-      <c r="QA48" s="27"/>
-      <c r="QB48" s="27"/>
-      <c r="QC48" s="27"/>
-      <c r="QD48" s="27"/>
-      <c r="QE48" s="27"/>
-      <c r="QF48" s="27"/>
-      <c r="QG48" s="27"/>
-      <c r="QH48" s="27"/>
-      <c r="QI48" s="27"/>
-      <c r="QJ48" s="27"/>
-      <c r="QK48" s="27"/>
-      <c r="QL48" s="27"/>
-      <c r="QM48" s="27"/>
-      <c r="QN48" s="27"/>
-      <c r="QO48" s="27"/>
-      <c r="QP48" s="27"/>
-      <c r="QQ48" s="27"/>
-      <c r="QR48" s="27"/>
-      <c r="QS48" s="27"/>
-      <c r="QT48" s="27"/>
-      <c r="QU48" s="27"/>
-      <c r="QV48" s="27"/>
-      <c r="QW48" s="27"/>
-      <c r="QX48" s="27"/>
-      <c r="QY48" s="27"/>
-      <c r="QZ48" s="27"/>
-      <c r="RA48" s="27"/>
-      <c r="RB48" s="27"/>
-      <c r="RC48" s="27"/>
-      <c r="RD48" s="27"/>
-      <c r="RE48" s="27"/>
-      <c r="RF48" s="27"/>
-      <c r="RG48" s="27"/>
-      <c r="RH48" s="27"/>
-      <c r="RI48" s="27"/>
-      <c r="RJ48" s="27"/>
-      <c r="RK48" s="27"/>
-      <c r="RL48" s="27"/>
-      <c r="RM48" s="27"/>
-      <c r="RN48" s="27"/>
-      <c r="RO48" s="27"/>
-      <c r="RP48" s="27"/>
-      <c r="RQ48" s="27"/>
-      <c r="RR48" s="27"/>
-      <c r="RS48" s="27"/>
-      <c r="RT48" s="27"/>
-      <c r="RU48" s="27"/>
-      <c r="RV48" s="27"/>
-      <c r="RW48" s="27"/>
-      <c r="RX48" s="27"/>
-      <c r="RY48" s="27"/>
-      <c r="RZ48" s="27"/>
-      <c r="SA48" s="27"/>
-      <c r="SB48" s="27"/>
-      <c r="SC48" s="27"/>
-      <c r="SD48" s="27"/>
-      <c r="SE48" s="27"/>
-      <c r="SF48" s="27"/>
-      <c r="SG48" s="27"/>
-      <c r="SH48" s="27"/>
-      <c r="SI48" s="27"/>
-      <c r="SJ48" s="27"/>
-      <c r="SK48" s="27"/>
-      <c r="SL48" s="27"/>
-      <c r="SM48" s="27"/>
-      <c r="SN48" s="27"/>
-      <c r="SO48" s="27"/>
-      <c r="SP48" s="27"/>
-      <c r="SQ48" s="27"/>
-      <c r="SR48" s="27"/>
-      <c r="SS48" s="27"/>
-      <c r="ST48" s="27"/>
-      <c r="SU48" s="27"/>
-      <c r="SV48" s="27"/>
-      <c r="SW48" s="27"/>
-      <c r="SX48" s="27"/>
-      <c r="SY48" s="27"/>
-      <c r="SZ48" s="27"/>
-      <c r="TA48" s="27"/>
-      <c r="TB48" s="27"/>
-      <c r="TC48" s="27"/>
-      <c r="TD48" s="27"/>
-      <c r="TE48" s="27"/>
-      <c r="TF48" s="27"/>
-      <c r="TG48" s="27"/>
-      <c r="TH48" s="27"/>
-      <c r="TI48" s="27"/>
-      <c r="TJ48" s="27"/>
-      <c r="TK48" s="27"/>
-      <c r="TL48" s="27"/>
-      <c r="TM48" s="27"/>
-      <c r="TN48" s="27"/>
-      <c r="TO48" s="27"/>
-      <c r="TP48" s="27"/>
-      <c r="TQ48" s="27"/>
-      <c r="TR48" s="27"/>
-      <c r="TS48" s="27"/>
-      <c r="TT48" s="27"/>
-      <c r="TU48" s="27"/>
-      <c r="TV48" s="27"/>
-      <c r="TW48" s="27"/>
-      <c r="TX48" s="27"/>
-      <c r="TY48" s="27"/>
-      <c r="TZ48" s="27"/>
-      <c r="UA48" s="27"/>
-      <c r="UB48" s="27"/>
-      <c r="UC48" s="27"/>
-      <c r="UD48" s="27"/>
-      <c r="UE48" s="27"/>
-      <c r="UF48" s="27"/>
-      <c r="UG48" s="27"/>
-      <c r="UH48" s="27"/>
-      <c r="UI48" s="27"/>
-      <c r="UJ48" s="27"/>
-      <c r="UK48" s="27"/>
-      <c r="UL48" s="27"/>
-      <c r="UM48" s="27"/>
-      <c r="UN48" s="27"/>
-      <c r="UO48" s="27"/>
-      <c r="UP48" s="27"/>
-      <c r="UQ48" s="27"/>
-      <c r="UR48" s="27"/>
-      <c r="US48" s="27"/>
-      <c r="UT48" s="27"/>
-      <c r="UU48" s="27"/>
-      <c r="UV48" s="27"/>
-      <c r="UW48" s="27"/>
-      <c r="UX48" s="27"/>
-      <c r="UY48" s="27"/>
-      <c r="UZ48" s="27"/>
-      <c r="VA48" s="27"/>
-      <c r="VB48" s="27"/>
-      <c r="VC48" s="27"/>
-      <c r="VD48" s="27"/>
-      <c r="VE48" s="27"/>
-      <c r="VF48" s="27"/>
-      <c r="VG48" s="27"/>
-      <c r="VH48" s="27"/>
-      <c r="VI48" s="27"/>
-      <c r="VJ48" s="27"/>
-      <c r="VK48" s="27"/>
-      <c r="VL48" s="27"/>
-      <c r="VM48" s="27"/>
-      <c r="VN48" s="27"/>
-      <c r="VO48" s="27"/>
-      <c r="VP48" s="27"/>
-      <c r="VQ48" s="27"/>
-      <c r="VR48" s="27"/>
-      <c r="VS48" s="27"/>
-      <c r="VT48" s="27"/>
-      <c r="VU48" s="27"/>
-      <c r="VV48" s="27"/>
-      <c r="VW48" s="27"/>
-      <c r="VX48" s="27"/>
-      <c r="VY48" s="27"/>
-      <c r="VZ48" s="27"/>
-      <c r="WA48" s="27"/>
-      <c r="WB48" s="27"/>
-      <c r="WC48" s="27"/>
-      <c r="WD48" s="27"/>
-      <c r="WE48" s="27"/>
-      <c r="WF48" s="27"/>
-      <c r="WG48" s="27"/>
-      <c r="WH48" s="27"/>
-      <c r="WI48" s="27"/>
-      <c r="WJ48" s="27"/>
-      <c r="WK48" s="27"/>
-      <c r="WL48" s="27"/>
-      <c r="WM48" s="27"/>
-      <c r="WN48" s="27"/>
-      <c r="WO48" s="27"/>
-      <c r="WP48" s="27"/>
-      <c r="WQ48" s="27"/>
-      <c r="WR48" s="27"/>
-      <c r="WS48" s="27"/>
-      <c r="WT48" s="27"/>
-      <c r="WU48" s="27"/>
-      <c r="WV48" s="27"/>
-      <c r="WW48" s="27"/>
-      <c r="WX48" s="27"/>
-      <c r="WY48" s="27"/>
-      <c r="WZ48" s="27"/>
-      <c r="XA48" s="27"/>
-      <c r="XB48" s="27"/>
-      <c r="XC48" s="27"/>
-      <c r="XD48" s="27"/>
-      <c r="XE48" s="27"/>
-      <c r="XF48" s="27"/>
-      <c r="XG48" s="27"/>
-      <c r="XH48" s="27"/>
-      <c r="XI48" s="27"/>
-      <c r="XJ48" s="27"/>
-      <c r="XK48" s="27"/>
-      <c r="XL48" s="27"/>
-      <c r="XM48" s="27"/>
-      <c r="XN48" s="27"/>
-      <c r="XO48" s="27"/>
-      <c r="XP48" s="27"/>
-      <c r="XQ48" s="27"/>
-      <c r="XR48" s="27"/>
-      <c r="XS48" s="27"/>
-      <c r="XT48" s="27"/>
-      <c r="XU48" s="27"/>
-      <c r="XV48" s="27"/>
-      <c r="XW48" s="27"/>
-      <c r="XX48" s="27"/>
-      <c r="XY48" s="27"/>
-      <c r="XZ48" s="27"/>
-      <c r="YA48" s="27"/>
-      <c r="YB48" s="27"/>
-      <c r="YC48" s="27"/>
-      <c r="YD48" s="27"/>
-      <c r="YE48" s="27"/>
-      <c r="YF48" s="27"/>
-      <c r="YG48" s="27"/>
-      <c r="YH48" s="27"/>
-      <c r="YI48" s="27"/>
-      <c r="YJ48" s="27"/>
-      <c r="YK48" s="27"/>
-      <c r="YL48" s="27"/>
-      <c r="YM48" s="27"/>
-      <c r="YN48" s="27"/>
-      <c r="YO48" s="27"/>
-      <c r="YP48" s="27"/>
-      <c r="YQ48" s="27"/>
-      <c r="YR48" s="27"/>
-      <c r="YS48" s="27"/>
-      <c r="YT48" s="27"/>
-      <c r="YU48" s="27"/>
-      <c r="YV48" s="27"/>
-      <c r="YW48" s="27"/>
-      <c r="YX48" s="27"/>
-      <c r="YY48" s="27"/>
-      <c r="YZ48" s="27"/>
-      <c r="ZA48" s="27"/>
-      <c r="ZB48" s="27"/>
-      <c r="ZC48" s="27"/>
-      <c r="ZD48" s="27"/>
-      <c r="ZE48" s="27"/>
-      <c r="ZF48" s="27"/>
-      <c r="ZG48" s="27"/>
-      <c r="ZH48" s="27"/>
-      <c r="ZI48" s="27"/>
-      <c r="ZJ48" s="27"/>
-      <c r="ZK48" s="27"/>
-      <c r="ZL48" s="27"/>
-      <c r="ZM48" s="27"/>
-      <c r="ZN48" s="27"/>
-      <c r="ZO48" s="27"/>
-      <c r="ZP48" s="27"/>
-      <c r="ZQ48" s="27"/>
-      <c r="ZR48" s="27"/>
-      <c r="ZS48" s="27"/>
-      <c r="ZT48" s="27"/>
-      <c r="ZU48" s="27"/>
-      <c r="ZV48" s="27"/>
-      <c r="ZW48" s="27"/>
-      <c r="ZX48" s="27"/>
-      <c r="ZY48" s="27"/>
-      <c r="ZZ48" s="27"/>
-      <c r="AAA48" s="27"/>
-      <c r="AAB48" s="27"/>
-      <c r="AAC48" s="27"/>
-      <c r="AAD48" s="27"/>
-      <c r="AAE48" s="27"/>
-      <c r="AAF48" s="27"/>
-      <c r="AAG48" s="27"/>
-      <c r="AAH48" s="27"/>
-      <c r="AAI48" s="27"/>
-      <c r="AAJ48" s="27"/>
-      <c r="AAK48" s="27"/>
-      <c r="AAL48" s="27"/>
-      <c r="AAM48" s="27"/>
-      <c r="AAN48" s="27"/>
-      <c r="AAO48" s="27"/>
-      <c r="AAP48" s="27"/>
-      <c r="AAQ48" s="27"/>
-      <c r="AAR48" s="27"/>
-      <c r="AAS48" s="27"/>
-      <c r="AAT48" s="27"/>
-      <c r="AAU48" s="27"/>
-      <c r="AAV48" s="27"/>
-      <c r="AAW48" s="27"/>
-      <c r="AAX48" s="27"/>
-      <c r="AAY48" s="27"/>
-      <c r="AAZ48" s="27"/>
-      <c r="ABA48" s="27"/>
-      <c r="ABB48" s="27"/>
-      <c r="ABC48" s="27"/>
-      <c r="ABD48" s="27"/>
-      <c r="ABE48" s="27"/>
-      <c r="ABF48" s="27"/>
-      <c r="ABG48" s="27"/>
-      <c r="ABH48" s="27"/>
-      <c r="ABI48" s="27"/>
-      <c r="ABJ48" s="27"/>
-      <c r="ABK48" s="27"/>
-      <c r="ABL48" s="27"/>
-      <c r="ABM48" s="27"/>
-      <c r="ABN48" s="27"/>
-      <c r="ABO48" s="27"/>
-      <c r="ABP48" s="27"/>
-      <c r="ABQ48" s="27"/>
-      <c r="ABR48" s="27"/>
-      <c r="ABS48" s="27"/>
-      <c r="ABT48" s="27"/>
-      <c r="ABU48" s="27"/>
-      <c r="ABV48" s="27"/>
-      <c r="ABW48" s="27"/>
-      <c r="ABX48" s="27"/>
-      <c r="ABY48" s="27"/>
-      <c r="ABZ48" s="27"/>
-      <c r="ACA48" s="27"/>
-      <c r="ACB48" s="27"/>
-      <c r="ACC48" s="27"/>
-      <c r="ACD48" s="27"/>
-      <c r="ACE48" s="27"/>
-      <c r="ACF48" s="27"/>
-      <c r="ACG48" s="27"/>
-      <c r="ACH48" s="27"/>
-      <c r="ACI48" s="27"/>
-      <c r="ACJ48" s="27"/>
-      <c r="ACK48" s="27"/>
-      <c r="ACL48" s="27"/>
-      <c r="ACM48" s="27"/>
-      <c r="ACN48" s="27"/>
-      <c r="ACO48" s="27"/>
-      <c r="ACP48" s="27"/>
-      <c r="ACQ48" s="27"/>
-      <c r="ACR48" s="27"/>
-      <c r="ACS48" s="27"/>
-      <c r="ACT48" s="27"/>
-      <c r="ACU48" s="27"/>
-      <c r="ACV48" s="27"/>
-      <c r="ACW48" s="27"/>
-      <c r="ACX48" s="27"/>
-      <c r="ACY48" s="27"/>
-      <c r="ACZ48" s="27"/>
-      <c r="ADA48" s="27"/>
-      <c r="ADB48" s="27"/>
-      <c r="ADC48" s="27"/>
-      <c r="ADD48" s="27"/>
-      <c r="ADE48" s="27"/>
-      <c r="ADF48" s="27"/>
-      <c r="ADG48" s="27"/>
-      <c r="ADH48" s="27"/>
-      <c r="ADI48" s="27"/>
-      <c r="ADJ48" s="27"/>
-      <c r="ADK48" s="27"/>
-      <c r="ADL48" s="27"/>
-      <c r="ADM48" s="27"/>
-      <c r="ADN48" s="27"/>
-      <c r="ADO48" s="27"/>
-      <c r="ADP48" s="27"/>
-      <c r="ADQ48" s="27"/>
-      <c r="ADR48" s="27"/>
-      <c r="ADS48" s="27"/>
-      <c r="ADT48" s="27"/>
-      <c r="ADU48" s="27"/>
-      <c r="ADV48" s="27"/>
-      <c r="ADW48" s="27"/>
-      <c r="ADX48" s="27"/>
-      <c r="ADY48" s="27"/>
-      <c r="ADZ48" s="27"/>
-      <c r="AEA48" s="27"/>
-      <c r="AEB48" s="27"/>
-      <c r="AEC48" s="27"/>
-      <c r="AED48" s="27"/>
-      <c r="AEE48" s="27"/>
-      <c r="AEF48" s="27"/>
-      <c r="AEG48" s="27"/>
-      <c r="AEH48" s="27"/>
-      <c r="AEI48" s="27"/>
-      <c r="AEJ48" s="27"/>
-      <c r="AEK48" s="27"/>
-      <c r="AEL48" s="27"/>
-      <c r="AEM48" s="27"/>
-      <c r="AEN48" s="27"/>
-      <c r="AEO48" s="27"/>
-      <c r="AEP48" s="27"/>
-      <c r="AEQ48" s="27"/>
-      <c r="AER48" s="27"/>
-      <c r="AES48" s="27"/>
-      <c r="AET48" s="27"/>
-      <c r="AEU48" s="27"/>
-      <c r="AEV48" s="27"/>
-      <c r="AEW48" s="27"/>
-      <c r="AEX48" s="27"/>
-      <c r="AEY48" s="27"/>
-      <c r="AEZ48" s="27"/>
-      <c r="AFA48" s="27"/>
-      <c r="AFB48" s="27"/>
-      <c r="AFC48" s="27"/>
-      <c r="AFD48" s="27"/>
-      <c r="AFE48" s="27"/>
-      <c r="AFF48" s="27"/>
-      <c r="AFG48" s="27"/>
-      <c r="AFH48" s="27"/>
-      <c r="AFI48" s="27"/>
-      <c r="AFJ48" s="27"/>
-      <c r="AFK48" s="27"/>
-      <c r="AFL48" s="27"/>
-      <c r="AFM48" s="27"/>
-      <c r="AFN48" s="27"/>
-      <c r="AFO48" s="27"/>
-      <c r="AFP48" s="27"/>
-      <c r="AFQ48" s="27"/>
-      <c r="AFR48" s="27"/>
-      <c r="AFS48" s="27"/>
-      <c r="AFT48" s="27"/>
-      <c r="AFU48" s="27"/>
-      <c r="AFV48" s="27"/>
-      <c r="AFW48" s="27"/>
-      <c r="AFX48" s="27"/>
-      <c r="AFY48" s="27"/>
-      <c r="AFZ48" s="27"/>
-      <c r="AGA48" s="27"/>
-      <c r="AGB48" s="27"/>
-      <c r="AGC48" s="27"/>
-      <c r="AGD48" s="27"/>
-      <c r="AGE48" s="27"/>
-      <c r="AGF48" s="27"/>
-      <c r="AGG48" s="27"/>
-      <c r="AGH48" s="27"/>
-      <c r="AGI48" s="27"/>
-      <c r="AGJ48" s="27"/>
-      <c r="AGK48" s="27"/>
-      <c r="AGL48" s="27"/>
-      <c r="AGM48" s="27"/>
-      <c r="AGN48" s="27"/>
-      <c r="AGO48" s="27"/>
-      <c r="AGP48" s="27"/>
-      <c r="AGQ48" s="27"/>
-      <c r="AGR48" s="27"/>
-      <c r="AGS48" s="27"/>
-      <c r="AGT48" s="27"/>
-      <c r="AGU48" s="27"/>
-      <c r="AGV48" s="27"/>
-      <c r="AGW48" s="27"/>
-      <c r="AGX48" s="27"/>
-      <c r="AGY48" s="27"/>
-      <c r="AGZ48" s="27"/>
-      <c r="AHA48" s="27"/>
-      <c r="AHB48" s="27"/>
-      <c r="AHC48" s="27"/>
-      <c r="AHD48" s="27"/>
-      <c r="AHE48" s="27"/>
-      <c r="AHF48" s="27"/>
-      <c r="AHG48" s="27"/>
-      <c r="AHH48" s="27"/>
-      <c r="AHI48" s="27"/>
-      <c r="AHJ48" s="27"/>
-      <c r="AHK48" s="27"/>
-      <c r="AHL48" s="27"/>
-      <c r="AHM48" s="27"/>
-      <c r="AHN48" s="27"/>
-      <c r="AHO48" s="27"/>
-      <c r="AHP48" s="27"/>
-      <c r="AHQ48" s="27"/>
-      <c r="AHR48" s="27"/>
-      <c r="AHS48" s="27"/>
-      <c r="AHT48" s="27"/>
-      <c r="AHU48" s="27"/>
-      <c r="AHV48" s="27"/>
-      <c r="AHW48" s="27"/>
-      <c r="AHX48" s="27"/>
-      <c r="AHY48" s="27"/>
-      <c r="AHZ48" s="27"/>
-      <c r="AIA48" s="27"/>
-      <c r="AIB48" s="27"/>
-      <c r="AIC48" s="27"/>
-      <c r="AID48" s="27"/>
-      <c r="AIE48" s="27"/>
-      <c r="AIF48" s="27"/>
-      <c r="AIG48" s="27"/>
-      <c r="AIH48" s="27"/>
-      <c r="AII48" s="27"/>
-      <c r="AIJ48" s="27"/>
-      <c r="AIK48" s="27"/>
-      <c r="AIL48" s="27"/>
-      <c r="AIM48" s="27"/>
-      <c r="AIN48" s="27"/>
-      <c r="AIO48" s="27"/>
-      <c r="AIP48" s="27"/>
-      <c r="AIQ48" s="27"/>
-      <c r="AIR48" s="27"/>
-      <c r="AIS48" s="27"/>
-      <c r="AIT48" s="27"/>
-      <c r="AIU48" s="27"/>
-      <c r="AIV48" s="27"/>
-      <c r="AIW48" s="27"/>
-      <c r="AIX48" s="27"/>
-      <c r="AIY48" s="27"/>
-      <c r="AIZ48" s="27"/>
-      <c r="AJA48" s="27"/>
-      <c r="AJB48" s="27"/>
-      <c r="AJC48" s="27"/>
-      <c r="AJD48" s="27"/>
-      <c r="AJE48" s="27"/>
-      <c r="AJF48" s="27"/>
-      <c r="AJG48" s="27"/>
-      <c r="AJH48" s="27"/>
-      <c r="AJI48" s="27"/>
-      <c r="AJJ48" s="27"/>
-      <c r="AJK48" s="27"/>
-      <c r="AJL48" s="27"/>
-      <c r="AJM48" s="27"/>
-      <c r="AJN48" s="27"/>
-      <c r="AJO48" s="27"/>
-      <c r="AJP48" s="27"/>
-      <c r="AJQ48" s="27"/>
-      <c r="AJR48" s="27"/>
-      <c r="AJS48" s="27"/>
-      <c r="AJT48" s="27"/>
-      <c r="AJU48" s="27"/>
-      <c r="AJV48" s="27"/>
-      <c r="AJW48" s="27"/>
-      <c r="AJX48" s="27"/>
-      <c r="AJY48" s="27"/>
-      <c r="AJZ48" s="27"/>
-      <c r="AKA48" s="27"/>
-      <c r="AKB48" s="27"/>
-      <c r="AKC48" s="27"/>
-      <c r="AKD48" s="27"/>
-      <c r="AKE48" s="27"/>
-      <c r="AKF48" s="27"/>
-      <c r="AKG48" s="27"/>
-      <c r="AKH48" s="27"/>
-      <c r="AKI48" s="27"/>
-      <c r="AKJ48" s="27"/>
-      <c r="AKK48" s="27"/>
-      <c r="AKL48" s="27"/>
-      <c r="AKM48" s="27"/>
-      <c r="AKN48" s="27"/>
-      <c r="AKO48" s="27"/>
-      <c r="AKP48" s="27"/>
-      <c r="AKQ48" s="27"/>
-      <c r="AKR48" s="27"/>
-      <c r="AKS48" s="27"/>
-      <c r="AKT48" s="27"/>
-      <c r="AKU48" s="27"/>
-      <c r="AKV48" s="27"/>
-      <c r="AKW48" s="27"/>
-      <c r="AKX48" s="27"/>
-      <c r="AKY48" s="27"/>
-      <c r="AKZ48" s="27"/>
-      <c r="ALA48" s="27"/>
-      <c r="ALB48" s="27"/>
-      <c r="ALC48" s="27"/>
-      <c r="ALD48" s="27"/>
-      <c r="ALE48" s="27"/>
-      <c r="ALF48" s="27"/>
-      <c r="ALG48" s="27"/>
-      <c r="ALH48" s="27"/>
-      <c r="ALI48" s="27"/>
-      <c r="ALJ48" s="27"/>
-      <c r="ALK48" s="27"/>
-      <c r="ALL48" s="27"/>
-      <c r="ALM48" s="27"/>
-      <c r="ALN48" s="27"/>
-      <c r="ALO48" s="27"/>
-      <c r="ALP48" s="27"/>
-      <c r="ALQ48" s="27"/>
-      <c r="ALR48" s="27"/>
-      <c r="ALS48" s="27"/>
-      <c r="ALT48" s="27"/>
-      <c r="ALU48" s="27"/>
-      <c r="ALV48" s="27"/>
-      <c r="ALW48" s="27"/>
-      <c r="ALX48" s="27"/>
-      <c r="ALY48" s="27"/>
-      <c r="ALZ48" s="27"/>
-      <c r="AMA48" s="27"/>
-      <c r="AMB48" s="27"/>
-      <c r="AMC48" s="27"/>
-      <c r="AMD48" s="27"/>
-      <c r="AME48" s="27"/>
-      <c r="AMF48" s="27"/>
-      <c r="AMG48" s="27"/>
-      <c r="AMH48" s="27"/>
-      <c r="AMI48" s="27"/>
-      <c r="AMJ48" s="27"/>
-      <c r="AMK48" s="27"/>
-    </row>
-    <row r="49" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="49" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="5" t="s">
         <v>210</v>
       </c>
@@ -6104,10 +4095,8 @@
       <c r="T49" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="U49" s="23"/>
-    </row>
-    <row r="50" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="23"/>
+    </row>
+    <row r="50" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="5" t="s">
         <v>279</v>
       </c>
@@ -6153,7 +4142,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="5" t="s">
         <v>214</v>
       </c>
@@ -6199,7 +4188,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:20" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="5" t="s">
         <v>245</v>
       </c>
@@ -6245,7 +4234,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="32" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:20" ht="32" x14ac:dyDescent="0.2">
       <c r="B53" s="5" t="s">
         <v>242</v>
       </c>
@@ -6291,7 +4280,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="32" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:20" ht="32" x14ac:dyDescent="0.2">
       <c r="B54" s="5" t="s">
         <v>235</v>
       </c>
@@ -6338,8 +4327,8 @@
         <v>239</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="58" spans="1:21" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="58" spans="2:20" ht="16" x14ac:dyDescent="0.2">
       <c r="B58" s="5" t="s">
         <v>186</v>
       </c>
@@ -6378,1072 +4367,49 @@
         <v>189</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="61" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="62" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B62" s="32" t="s">
+    <row r="60" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="61" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="62" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B62" s="30" t="s">
         <v>190</v>
       </c>
-      <c r="C62" s="32"/>
-    </row>
-    <row r="63" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B63" s="33" t="s">
+      <c r="C62" s="30"/>
+    </row>
+    <row r="63" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B63" s="31" t="s">
         <v>191</v>
       </c>
-      <c r="C63" s="33"/>
-    </row>
-    <row r="64" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B64" s="33" t="s">
+      <c r="C63" s="31"/>
+    </row>
+    <row r="64" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B64" s="31" t="s">
         <v>192</v>
       </c>
-      <c r="C64" s="33"/>
-    </row>
-    <row r="65" spans="1:1025" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B65" s="34" t="s">
+      <c r="C64" s="31"/>
+    </row>
+    <row r="65" spans="2:3" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B65" s="32" t="s">
         <v>193</v>
       </c>
-      <c r="C65" s="34"/>
-    </row>
-    <row r="66" spans="1:1025" x14ac:dyDescent="0.2">
-      <c r="B66" s="34" t="s">
+      <c r="C65" s="32"/>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B66" s="32" t="s">
         <v>194</v>
       </c>
-      <c r="C66" s="34"/>
-    </row>
-    <row r="67" spans="1:1025" x14ac:dyDescent="0.2">
-      <c r="A67" s="26"/>
-      <c r="B67" s="34" t="s">
+      <c r="C66" s="32"/>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B67" s="32" t="s">
         <v>259</v>
       </c>
-      <c r="C67" s="34"/>
-      <c r="D67" s="26"/>
-      <c r="E67" s="26"/>
-      <c r="F67" s="26"/>
-      <c r="G67" s="26"/>
-      <c r="H67" s="26"/>
-      <c r="I67" s="26"/>
-      <c r="J67" s="26"/>
-      <c r="K67" s="26"/>
-      <c r="L67" s="26"/>
-      <c r="M67" s="26"/>
-      <c r="N67" s="26"/>
-      <c r="O67" s="26"/>
-      <c r="P67" s="26"/>
-      <c r="Q67" s="26"/>
-      <c r="R67" s="26"/>
-      <c r="S67" s="26"/>
-      <c r="T67" s="26"/>
-      <c r="U67" s="26"/>
-      <c r="V67" s="26"/>
-      <c r="W67" s="26"/>
-      <c r="X67" s="26"/>
-      <c r="Y67" s="26"/>
-      <c r="Z67" s="26"/>
-      <c r="AA67" s="26"/>
-      <c r="AB67" s="26"/>
-      <c r="AC67" s="26"/>
-      <c r="AD67" s="26"/>
-      <c r="AE67" s="26"/>
-      <c r="AF67" s="26"/>
-      <c r="AG67" s="26"/>
-      <c r="AH67" s="26"/>
-      <c r="AI67" s="26"/>
-      <c r="AJ67" s="26"/>
-      <c r="AK67" s="26"/>
-      <c r="AL67" s="26"/>
-      <c r="AM67" s="26"/>
-      <c r="AN67" s="26"/>
-      <c r="AO67" s="26"/>
-      <c r="AP67" s="26"/>
-      <c r="AQ67" s="26"/>
-      <c r="AR67" s="26"/>
-      <c r="AS67" s="26"/>
-      <c r="AT67" s="26"/>
-      <c r="AU67" s="26"/>
-      <c r="AV67" s="26"/>
-      <c r="AW67" s="26"/>
-      <c r="AX67" s="26"/>
-      <c r="AY67" s="26"/>
-      <c r="AZ67" s="26"/>
-      <c r="BA67" s="26"/>
-      <c r="BB67" s="26"/>
-      <c r="BC67" s="26"/>
-      <c r="BD67" s="26"/>
-      <c r="BE67" s="26"/>
-      <c r="BF67" s="26"/>
-      <c r="BG67" s="26"/>
-      <c r="BH67" s="26"/>
-      <c r="BI67" s="26"/>
-      <c r="BJ67" s="26"/>
-      <c r="BK67" s="26"/>
-      <c r="BL67" s="26"/>
-      <c r="BM67" s="26"/>
-      <c r="BN67" s="26"/>
-      <c r="BO67" s="26"/>
-      <c r="BP67" s="26"/>
-      <c r="BQ67" s="26"/>
-      <c r="BR67" s="26"/>
-      <c r="BS67" s="26"/>
-      <c r="BT67" s="26"/>
-      <c r="BU67" s="26"/>
-      <c r="BV67" s="26"/>
-      <c r="BW67" s="26"/>
-      <c r="BX67" s="26"/>
-      <c r="BY67" s="26"/>
-      <c r="BZ67" s="26"/>
-      <c r="CA67" s="26"/>
-      <c r="CB67" s="26"/>
-      <c r="CC67" s="26"/>
-      <c r="CD67" s="26"/>
-      <c r="CE67" s="26"/>
-      <c r="CF67" s="26"/>
-      <c r="CG67" s="26"/>
-      <c r="CH67" s="26"/>
-      <c r="CI67" s="26"/>
-      <c r="CJ67" s="26"/>
-      <c r="CK67" s="26"/>
-      <c r="CL67" s="26"/>
-      <c r="CM67" s="26"/>
-      <c r="CN67" s="26"/>
-      <c r="CO67" s="26"/>
-      <c r="CP67" s="26"/>
-      <c r="CQ67" s="26"/>
-      <c r="CR67" s="26"/>
-      <c r="CS67" s="26"/>
-      <c r="CT67" s="26"/>
-      <c r="CU67" s="26"/>
-      <c r="CV67" s="26"/>
-      <c r="CW67" s="26"/>
-      <c r="CX67" s="26"/>
-      <c r="CY67" s="26"/>
-      <c r="CZ67" s="26"/>
-      <c r="DA67" s="26"/>
-      <c r="DB67" s="26"/>
-      <c r="DC67" s="26"/>
-      <c r="DD67" s="26"/>
-      <c r="DE67" s="26"/>
-      <c r="DF67" s="26"/>
-      <c r="DG67" s="26"/>
-      <c r="DH67" s="26"/>
-      <c r="DI67" s="26"/>
-      <c r="DJ67" s="26"/>
-      <c r="DK67" s="26"/>
-      <c r="DL67" s="26"/>
-      <c r="DM67" s="26"/>
-      <c r="DN67" s="26"/>
-      <c r="DO67" s="26"/>
-      <c r="DP67" s="26"/>
-      <c r="DQ67" s="26"/>
-      <c r="DR67" s="26"/>
-      <c r="DS67" s="26"/>
-      <c r="DT67" s="26"/>
-      <c r="DU67" s="26"/>
-      <c r="DV67" s="26"/>
-      <c r="DW67" s="26"/>
-      <c r="DX67" s="26"/>
-      <c r="DY67" s="26"/>
-      <c r="DZ67" s="26"/>
-      <c r="EA67" s="26"/>
-      <c r="EB67" s="26"/>
-      <c r="EC67" s="26"/>
-      <c r="ED67" s="26"/>
-      <c r="EE67" s="26"/>
-      <c r="EF67" s="26"/>
-      <c r="EG67" s="26"/>
-      <c r="EH67" s="26"/>
-      <c r="EI67" s="26"/>
-      <c r="EJ67" s="26"/>
-      <c r="EK67" s="26"/>
-      <c r="EL67" s="26"/>
-      <c r="EM67" s="26"/>
-      <c r="EN67" s="26"/>
-      <c r="EO67" s="26"/>
-      <c r="EP67" s="26"/>
-      <c r="EQ67" s="26"/>
-      <c r="ER67" s="26"/>
-      <c r="ES67" s="26"/>
-      <c r="ET67" s="26"/>
-      <c r="EU67" s="26"/>
-      <c r="EV67" s="26"/>
-      <c r="EW67" s="26"/>
-      <c r="EX67" s="26"/>
-      <c r="EY67" s="26"/>
-      <c r="EZ67" s="26"/>
-      <c r="FA67" s="26"/>
-      <c r="FB67" s="26"/>
-      <c r="FC67" s="26"/>
-      <c r="FD67" s="26"/>
-      <c r="FE67" s="26"/>
-      <c r="FF67" s="26"/>
-      <c r="FG67" s="26"/>
-      <c r="FH67" s="26"/>
-      <c r="FI67" s="26"/>
-      <c r="FJ67" s="26"/>
-      <c r="FK67" s="26"/>
-      <c r="FL67" s="26"/>
-      <c r="FM67" s="26"/>
-      <c r="FN67" s="26"/>
-      <c r="FO67" s="26"/>
-      <c r="FP67" s="26"/>
-      <c r="FQ67" s="26"/>
-      <c r="FR67" s="26"/>
-      <c r="FS67" s="26"/>
-      <c r="FT67" s="26"/>
-      <c r="FU67" s="26"/>
-      <c r="FV67" s="26"/>
-      <c r="FW67" s="26"/>
-      <c r="FX67" s="26"/>
-      <c r="FY67" s="26"/>
-      <c r="FZ67" s="26"/>
-      <c r="GA67" s="26"/>
-      <c r="GB67" s="26"/>
-      <c r="GC67" s="26"/>
-      <c r="GD67" s="26"/>
-      <c r="GE67" s="26"/>
-      <c r="GF67" s="26"/>
-      <c r="GG67" s="26"/>
-      <c r="GH67" s="26"/>
-      <c r="GI67" s="26"/>
-      <c r="GJ67" s="26"/>
-      <c r="GK67" s="26"/>
-      <c r="GL67" s="26"/>
-      <c r="GM67" s="26"/>
-      <c r="GN67" s="26"/>
-      <c r="GO67" s="26"/>
-      <c r="GP67" s="26"/>
-      <c r="GQ67" s="26"/>
-      <c r="GR67" s="26"/>
-      <c r="GS67" s="26"/>
-      <c r="GT67" s="26"/>
-      <c r="GU67" s="26"/>
-      <c r="GV67" s="26"/>
-      <c r="GW67" s="26"/>
-      <c r="GX67" s="26"/>
-      <c r="GY67" s="26"/>
-      <c r="GZ67" s="26"/>
-      <c r="HA67" s="26"/>
-      <c r="HB67" s="26"/>
-      <c r="HC67" s="26"/>
-      <c r="HD67" s="26"/>
-      <c r="HE67" s="26"/>
-      <c r="HF67" s="26"/>
-      <c r="HG67" s="26"/>
-      <c r="HH67" s="26"/>
-      <c r="HI67" s="26"/>
-      <c r="HJ67" s="26"/>
-      <c r="HK67" s="26"/>
-      <c r="HL67" s="26"/>
-      <c r="HM67" s="26"/>
-      <c r="HN67" s="26"/>
-      <c r="HO67" s="26"/>
-      <c r="HP67" s="26"/>
-      <c r="HQ67" s="26"/>
-      <c r="HR67" s="26"/>
-      <c r="HS67" s="26"/>
-      <c r="HT67" s="26"/>
-      <c r="HU67" s="26"/>
-      <c r="HV67" s="26"/>
-      <c r="HW67" s="26"/>
-      <c r="HX67" s="26"/>
-      <c r="HY67" s="26"/>
-      <c r="HZ67" s="26"/>
-      <c r="IA67" s="26"/>
-      <c r="IB67" s="26"/>
-      <c r="IC67" s="26"/>
-      <c r="ID67" s="26"/>
-      <c r="IE67" s="26"/>
-      <c r="IF67" s="26"/>
-      <c r="IG67" s="26"/>
-      <c r="IH67" s="26"/>
-      <c r="II67" s="26"/>
-      <c r="IJ67" s="26"/>
-      <c r="IK67" s="26"/>
-      <c r="IL67" s="26"/>
-      <c r="IM67" s="26"/>
-      <c r="IN67" s="26"/>
-      <c r="IO67" s="26"/>
-      <c r="IP67" s="26"/>
-      <c r="IQ67" s="26"/>
-      <c r="IR67" s="26"/>
-      <c r="IS67" s="26"/>
-      <c r="IT67" s="26"/>
-      <c r="IU67" s="26"/>
-      <c r="IV67" s="26"/>
-      <c r="IW67" s="26"/>
-      <c r="IX67" s="26"/>
-      <c r="IY67" s="26"/>
-      <c r="IZ67" s="26"/>
-      <c r="JA67" s="26"/>
-      <c r="JB67" s="26"/>
-      <c r="JC67" s="26"/>
-      <c r="JD67" s="26"/>
-      <c r="JE67" s="26"/>
-      <c r="JF67" s="26"/>
-      <c r="JG67" s="26"/>
-      <c r="JH67" s="26"/>
-      <c r="JI67" s="26"/>
-      <c r="JJ67" s="26"/>
-      <c r="JK67" s="26"/>
-      <c r="JL67" s="26"/>
-      <c r="JM67" s="26"/>
-      <c r="JN67" s="26"/>
-      <c r="JO67" s="26"/>
-      <c r="JP67" s="26"/>
-      <c r="JQ67" s="26"/>
-      <c r="JR67" s="26"/>
-      <c r="JS67" s="26"/>
-      <c r="JT67" s="26"/>
-      <c r="JU67" s="26"/>
-      <c r="JV67" s="26"/>
-      <c r="JW67" s="26"/>
-      <c r="JX67" s="26"/>
-      <c r="JY67" s="26"/>
-      <c r="JZ67" s="26"/>
-      <c r="KA67" s="26"/>
-      <c r="KB67" s="26"/>
-      <c r="KC67" s="26"/>
-      <c r="KD67" s="26"/>
-      <c r="KE67" s="26"/>
-      <c r="KF67" s="26"/>
-      <c r="KG67" s="26"/>
-      <c r="KH67" s="26"/>
-      <c r="KI67" s="26"/>
-      <c r="KJ67" s="26"/>
-      <c r="KK67" s="26"/>
-      <c r="KL67" s="26"/>
-      <c r="KM67" s="26"/>
-      <c r="KN67" s="26"/>
-      <c r="KO67" s="26"/>
-      <c r="KP67" s="26"/>
-      <c r="KQ67" s="26"/>
-      <c r="KR67" s="26"/>
-      <c r="KS67" s="26"/>
-      <c r="KT67" s="26"/>
-      <c r="KU67" s="26"/>
-      <c r="KV67" s="26"/>
-      <c r="KW67" s="26"/>
-      <c r="KX67" s="26"/>
-      <c r="KY67" s="26"/>
-      <c r="KZ67" s="26"/>
-      <c r="LA67" s="26"/>
-      <c r="LB67" s="26"/>
-      <c r="LC67" s="26"/>
-      <c r="LD67" s="26"/>
-      <c r="LE67" s="26"/>
-      <c r="LF67" s="26"/>
-      <c r="LG67" s="26"/>
-      <c r="LH67" s="26"/>
-      <c r="LI67" s="26"/>
-      <c r="LJ67" s="26"/>
-      <c r="LK67" s="26"/>
-      <c r="LL67" s="26"/>
-      <c r="LM67" s="26"/>
-      <c r="LN67" s="26"/>
-      <c r="LO67" s="26"/>
-      <c r="LP67" s="26"/>
-      <c r="LQ67" s="26"/>
-      <c r="LR67" s="26"/>
-      <c r="LS67" s="26"/>
-      <c r="LT67" s="26"/>
-      <c r="LU67" s="26"/>
-      <c r="LV67" s="26"/>
-      <c r="LW67" s="26"/>
-      <c r="LX67" s="26"/>
-      <c r="LY67" s="26"/>
-      <c r="LZ67" s="26"/>
-      <c r="MA67" s="26"/>
-      <c r="MB67" s="26"/>
-      <c r="MC67" s="26"/>
-      <c r="MD67" s="26"/>
-      <c r="ME67" s="26"/>
-      <c r="MF67" s="26"/>
-      <c r="MG67" s="26"/>
-      <c r="MH67" s="26"/>
-      <c r="MI67" s="26"/>
-      <c r="MJ67" s="26"/>
-      <c r="MK67" s="26"/>
-      <c r="ML67" s="26"/>
-      <c r="MM67" s="26"/>
-      <c r="MN67" s="26"/>
-      <c r="MO67" s="26"/>
-      <c r="MP67" s="26"/>
-      <c r="MQ67" s="26"/>
-      <c r="MR67" s="26"/>
-      <c r="MS67" s="26"/>
-      <c r="MT67" s="26"/>
-      <c r="MU67" s="26"/>
-      <c r="MV67" s="26"/>
-      <c r="MW67" s="26"/>
-      <c r="MX67" s="26"/>
-      <c r="MY67" s="26"/>
-      <c r="MZ67" s="26"/>
-      <c r="NA67" s="26"/>
-      <c r="NB67" s="26"/>
-      <c r="NC67" s="26"/>
-      <c r="ND67" s="26"/>
-      <c r="NE67" s="26"/>
-      <c r="NF67" s="26"/>
-      <c r="NG67" s="26"/>
-      <c r="NH67" s="26"/>
-      <c r="NI67" s="26"/>
-      <c r="NJ67" s="26"/>
-      <c r="NK67" s="26"/>
-      <c r="NL67" s="26"/>
-      <c r="NM67" s="26"/>
-      <c r="NN67" s="26"/>
-      <c r="NO67" s="26"/>
-      <c r="NP67" s="26"/>
-      <c r="NQ67" s="26"/>
-      <c r="NR67" s="26"/>
-      <c r="NS67" s="26"/>
-      <c r="NT67" s="26"/>
-      <c r="NU67" s="26"/>
-      <c r="NV67" s="26"/>
-      <c r="NW67" s="26"/>
-      <c r="NX67" s="26"/>
-      <c r="NY67" s="26"/>
-      <c r="NZ67" s="26"/>
-      <c r="OA67" s="26"/>
-      <c r="OB67" s="26"/>
-      <c r="OC67" s="26"/>
-      <c r="OD67" s="26"/>
-      <c r="OE67" s="26"/>
-      <c r="OF67" s="26"/>
-      <c r="OG67" s="26"/>
-      <c r="OH67" s="26"/>
-      <c r="OI67" s="26"/>
-      <c r="OJ67" s="26"/>
-      <c r="OK67" s="26"/>
-      <c r="OL67" s="26"/>
-      <c r="OM67" s="26"/>
-      <c r="ON67" s="26"/>
-      <c r="OO67" s="26"/>
-      <c r="OP67" s="26"/>
-      <c r="OQ67" s="26"/>
-      <c r="OR67" s="26"/>
-      <c r="OS67" s="26"/>
-      <c r="OT67" s="26"/>
-      <c r="OU67" s="26"/>
-      <c r="OV67" s="26"/>
-      <c r="OW67" s="26"/>
-      <c r="OX67" s="26"/>
-      <c r="OY67" s="26"/>
-      <c r="OZ67" s="26"/>
-      <c r="PA67" s="26"/>
-      <c r="PB67" s="26"/>
-      <c r="PC67" s="26"/>
-      <c r="PD67" s="26"/>
-      <c r="PE67" s="26"/>
-      <c r="PF67" s="26"/>
-      <c r="PG67" s="26"/>
-      <c r="PH67" s="26"/>
-      <c r="PI67" s="26"/>
-      <c r="PJ67" s="26"/>
-      <c r="PK67" s="26"/>
-      <c r="PL67" s="26"/>
-      <c r="PM67" s="26"/>
-      <c r="PN67" s="26"/>
-      <c r="PO67" s="26"/>
-      <c r="PP67" s="26"/>
-      <c r="PQ67" s="26"/>
-      <c r="PR67" s="26"/>
-      <c r="PS67" s="26"/>
-      <c r="PT67" s="26"/>
-      <c r="PU67" s="26"/>
-      <c r="PV67" s="26"/>
-      <c r="PW67" s="26"/>
-      <c r="PX67" s="26"/>
-      <c r="PY67" s="26"/>
-      <c r="PZ67" s="26"/>
-      <c r="QA67" s="26"/>
-      <c r="QB67" s="26"/>
-      <c r="QC67" s="26"/>
-      <c r="QD67" s="26"/>
-      <c r="QE67" s="26"/>
-      <c r="QF67" s="26"/>
-      <c r="QG67" s="26"/>
-      <c r="QH67" s="26"/>
-      <c r="QI67" s="26"/>
-      <c r="QJ67" s="26"/>
-      <c r="QK67" s="26"/>
-      <c r="QL67" s="26"/>
-      <c r="QM67" s="26"/>
-      <c r="QN67" s="26"/>
-      <c r="QO67" s="26"/>
-      <c r="QP67" s="26"/>
-      <c r="QQ67" s="26"/>
-      <c r="QR67" s="26"/>
-      <c r="QS67" s="26"/>
-      <c r="QT67" s="26"/>
-      <c r="QU67" s="26"/>
-      <c r="QV67" s="26"/>
-      <c r="QW67" s="26"/>
-      <c r="QX67" s="26"/>
-      <c r="QY67" s="26"/>
-      <c r="QZ67" s="26"/>
-      <c r="RA67" s="26"/>
-      <c r="RB67" s="26"/>
-      <c r="RC67" s="26"/>
-      <c r="RD67" s="26"/>
-      <c r="RE67" s="26"/>
-      <c r="RF67" s="26"/>
-      <c r="RG67" s="26"/>
-      <c r="RH67" s="26"/>
-      <c r="RI67" s="26"/>
-      <c r="RJ67" s="26"/>
-      <c r="RK67" s="26"/>
-      <c r="RL67" s="26"/>
-      <c r="RM67" s="26"/>
-      <c r="RN67" s="26"/>
-      <c r="RO67" s="26"/>
-      <c r="RP67" s="26"/>
-      <c r="RQ67" s="26"/>
-      <c r="RR67" s="26"/>
-      <c r="RS67" s="26"/>
-      <c r="RT67" s="26"/>
-      <c r="RU67" s="26"/>
-      <c r="RV67" s="26"/>
-      <c r="RW67" s="26"/>
-      <c r="RX67" s="26"/>
-      <c r="RY67" s="26"/>
-      <c r="RZ67" s="26"/>
-      <c r="SA67" s="26"/>
-      <c r="SB67" s="26"/>
-      <c r="SC67" s="26"/>
-      <c r="SD67" s="26"/>
-      <c r="SE67" s="26"/>
-      <c r="SF67" s="26"/>
-      <c r="SG67" s="26"/>
-      <c r="SH67" s="26"/>
-      <c r="SI67" s="26"/>
-      <c r="SJ67" s="26"/>
-      <c r="SK67" s="26"/>
-      <c r="SL67" s="26"/>
-      <c r="SM67" s="26"/>
-      <c r="SN67" s="26"/>
-      <c r="SO67" s="26"/>
-      <c r="SP67" s="26"/>
-      <c r="SQ67" s="26"/>
-      <c r="SR67" s="26"/>
-      <c r="SS67" s="26"/>
-      <c r="ST67" s="26"/>
-      <c r="SU67" s="26"/>
-      <c r="SV67" s="26"/>
-      <c r="SW67" s="26"/>
-      <c r="SX67" s="26"/>
-      <c r="SY67" s="26"/>
-      <c r="SZ67" s="26"/>
-      <c r="TA67" s="26"/>
-      <c r="TB67" s="26"/>
-      <c r="TC67" s="26"/>
-      <c r="TD67" s="26"/>
-      <c r="TE67" s="26"/>
-      <c r="TF67" s="26"/>
-      <c r="TG67" s="26"/>
-      <c r="TH67" s="26"/>
-      <c r="TI67" s="26"/>
-      <c r="TJ67" s="26"/>
-      <c r="TK67" s="26"/>
-      <c r="TL67" s="26"/>
-      <c r="TM67" s="26"/>
-      <c r="TN67" s="26"/>
-      <c r="TO67" s="26"/>
-      <c r="TP67" s="26"/>
-      <c r="TQ67" s="26"/>
-      <c r="TR67" s="26"/>
-      <c r="TS67" s="26"/>
-      <c r="TT67" s="26"/>
-      <c r="TU67" s="26"/>
-      <c r="TV67" s="26"/>
-      <c r="TW67" s="26"/>
-      <c r="TX67" s="26"/>
-      <c r="TY67" s="26"/>
-      <c r="TZ67" s="26"/>
-      <c r="UA67" s="26"/>
-      <c r="UB67" s="26"/>
-      <c r="UC67" s="26"/>
-      <c r="UD67" s="26"/>
-      <c r="UE67" s="26"/>
-      <c r="UF67" s="26"/>
-      <c r="UG67" s="26"/>
-      <c r="UH67" s="26"/>
-      <c r="UI67" s="26"/>
-      <c r="UJ67" s="26"/>
-      <c r="UK67" s="26"/>
-      <c r="UL67" s="26"/>
-      <c r="UM67" s="26"/>
-      <c r="UN67" s="26"/>
-      <c r="UO67" s="26"/>
-      <c r="UP67" s="26"/>
-      <c r="UQ67" s="26"/>
-      <c r="UR67" s="26"/>
-      <c r="US67" s="26"/>
-      <c r="UT67" s="26"/>
-      <c r="UU67" s="26"/>
-      <c r="UV67" s="26"/>
-      <c r="UW67" s="26"/>
-      <c r="UX67" s="26"/>
-      <c r="UY67" s="26"/>
-      <c r="UZ67" s="26"/>
-      <c r="VA67" s="26"/>
-      <c r="VB67" s="26"/>
-      <c r="VC67" s="26"/>
-      <c r="VD67" s="26"/>
-      <c r="VE67" s="26"/>
-      <c r="VF67" s="26"/>
-      <c r="VG67" s="26"/>
-      <c r="VH67" s="26"/>
-      <c r="VI67" s="26"/>
-      <c r="VJ67" s="26"/>
-      <c r="VK67" s="26"/>
-      <c r="VL67" s="26"/>
-      <c r="VM67" s="26"/>
-      <c r="VN67" s="26"/>
-      <c r="VO67" s="26"/>
-      <c r="VP67" s="26"/>
-      <c r="VQ67" s="26"/>
-      <c r="VR67" s="26"/>
-      <c r="VS67" s="26"/>
-      <c r="VT67" s="26"/>
-      <c r="VU67" s="26"/>
-      <c r="VV67" s="26"/>
-      <c r="VW67" s="26"/>
-      <c r="VX67" s="26"/>
-      <c r="VY67" s="26"/>
-      <c r="VZ67" s="26"/>
-      <c r="WA67" s="26"/>
-      <c r="WB67" s="26"/>
-      <c r="WC67" s="26"/>
-      <c r="WD67" s="26"/>
-      <c r="WE67" s="26"/>
-      <c r="WF67" s="26"/>
-      <c r="WG67" s="26"/>
-      <c r="WH67" s="26"/>
-      <c r="WI67" s="26"/>
-      <c r="WJ67" s="26"/>
-      <c r="WK67" s="26"/>
-      <c r="WL67" s="26"/>
-      <c r="WM67" s="26"/>
-      <c r="WN67" s="26"/>
-      <c r="WO67" s="26"/>
-      <c r="WP67" s="26"/>
-      <c r="WQ67" s="26"/>
-      <c r="WR67" s="26"/>
-      <c r="WS67" s="26"/>
-      <c r="WT67" s="26"/>
-      <c r="WU67" s="26"/>
-      <c r="WV67" s="26"/>
-      <c r="WW67" s="26"/>
-      <c r="WX67" s="26"/>
-      <c r="WY67" s="26"/>
-      <c r="WZ67" s="26"/>
-      <c r="XA67" s="26"/>
-      <c r="XB67" s="26"/>
-      <c r="XC67" s="26"/>
-      <c r="XD67" s="26"/>
-      <c r="XE67" s="26"/>
-      <c r="XF67" s="26"/>
-      <c r="XG67" s="26"/>
-      <c r="XH67" s="26"/>
-      <c r="XI67" s="26"/>
-      <c r="XJ67" s="26"/>
-      <c r="XK67" s="26"/>
-      <c r="XL67" s="26"/>
-      <c r="XM67" s="26"/>
-      <c r="XN67" s="26"/>
-      <c r="XO67" s="26"/>
-      <c r="XP67" s="26"/>
-      <c r="XQ67" s="26"/>
-      <c r="XR67" s="26"/>
-      <c r="XS67" s="26"/>
-      <c r="XT67" s="26"/>
-      <c r="XU67" s="26"/>
-      <c r="XV67" s="26"/>
-      <c r="XW67" s="26"/>
-      <c r="XX67" s="26"/>
-      <c r="XY67" s="26"/>
-      <c r="XZ67" s="26"/>
-      <c r="YA67" s="26"/>
-      <c r="YB67" s="26"/>
-      <c r="YC67" s="26"/>
-      <c r="YD67" s="26"/>
-      <c r="YE67" s="26"/>
-      <c r="YF67" s="26"/>
-      <c r="YG67" s="26"/>
-      <c r="YH67" s="26"/>
-      <c r="YI67" s="26"/>
-      <c r="YJ67" s="26"/>
-      <c r="YK67" s="26"/>
-      <c r="YL67" s="26"/>
-      <c r="YM67" s="26"/>
-      <c r="YN67" s="26"/>
-      <c r="YO67" s="26"/>
-      <c r="YP67" s="26"/>
-      <c r="YQ67" s="26"/>
-      <c r="YR67" s="26"/>
-      <c r="YS67" s="26"/>
-      <c r="YT67" s="26"/>
-      <c r="YU67" s="26"/>
-      <c r="YV67" s="26"/>
-      <c r="YW67" s="26"/>
-      <c r="YX67" s="26"/>
-      <c r="YY67" s="26"/>
-      <c r="YZ67" s="26"/>
-      <c r="ZA67" s="26"/>
-      <c r="ZB67" s="26"/>
-      <c r="ZC67" s="26"/>
-      <c r="ZD67" s="26"/>
-      <c r="ZE67" s="26"/>
-      <c r="ZF67" s="26"/>
-      <c r="ZG67" s="26"/>
-      <c r="ZH67" s="26"/>
-      <c r="ZI67" s="26"/>
-      <c r="ZJ67" s="26"/>
-      <c r="ZK67" s="26"/>
-      <c r="ZL67" s="26"/>
-      <c r="ZM67" s="26"/>
-      <c r="ZN67" s="26"/>
-      <c r="ZO67" s="26"/>
-      <c r="ZP67" s="26"/>
-      <c r="ZQ67" s="26"/>
-      <c r="ZR67" s="26"/>
-      <c r="ZS67" s="26"/>
-      <c r="ZT67" s="26"/>
-      <c r="ZU67" s="26"/>
-      <c r="ZV67" s="26"/>
-      <c r="ZW67" s="26"/>
-      <c r="ZX67" s="26"/>
-      <c r="ZY67" s="26"/>
-      <c r="ZZ67" s="26"/>
-      <c r="AAA67" s="26"/>
-      <c r="AAB67" s="26"/>
-      <c r="AAC67" s="26"/>
-      <c r="AAD67" s="26"/>
-      <c r="AAE67" s="26"/>
-      <c r="AAF67" s="26"/>
-      <c r="AAG67" s="26"/>
-      <c r="AAH67" s="26"/>
-      <c r="AAI67" s="26"/>
-      <c r="AAJ67" s="26"/>
-      <c r="AAK67" s="26"/>
-      <c r="AAL67" s="26"/>
-      <c r="AAM67" s="26"/>
-      <c r="AAN67" s="26"/>
-      <c r="AAO67" s="26"/>
-      <c r="AAP67" s="26"/>
-      <c r="AAQ67" s="26"/>
-      <c r="AAR67" s="26"/>
-      <c r="AAS67" s="26"/>
-      <c r="AAT67" s="26"/>
-      <c r="AAU67" s="26"/>
-      <c r="AAV67" s="26"/>
-      <c r="AAW67" s="26"/>
-      <c r="AAX67" s="26"/>
-      <c r="AAY67" s="26"/>
-      <c r="AAZ67" s="26"/>
-      <c r="ABA67" s="26"/>
-      <c r="ABB67" s="26"/>
-      <c r="ABC67" s="26"/>
-      <c r="ABD67" s="26"/>
-      <c r="ABE67" s="26"/>
-      <c r="ABF67" s="26"/>
-      <c r="ABG67" s="26"/>
-      <c r="ABH67" s="26"/>
-      <c r="ABI67" s="26"/>
-      <c r="ABJ67" s="26"/>
-      <c r="ABK67" s="26"/>
-      <c r="ABL67" s="26"/>
-      <c r="ABM67" s="26"/>
-      <c r="ABN67" s="26"/>
-      <c r="ABO67" s="26"/>
-      <c r="ABP67" s="26"/>
-      <c r="ABQ67" s="26"/>
-      <c r="ABR67" s="26"/>
-      <c r="ABS67" s="26"/>
-      <c r="ABT67" s="26"/>
-      <c r="ABU67" s="26"/>
-      <c r="ABV67" s="26"/>
-      <c r="ABW67" s="26"/>
-      <c r="ABX67" s="26"/>
-      <c r="ABY67" s="26"/>
-      <c r="ABZ67" s="26"/>
-      <c r="ACA67" s="26"/>
-      <c r="ACB67" s="26"/>
-      <c r="ACC67" s="26"/>
-      <c r="ACD67" s="26"/>
-      <c r="ACE67" s="26"/>
-      <c r="ACF67" s="26"/>
-      <c r="ACG67" s="26"/>
-      <c r="ACH67" s="26"/>
-      <c r="ACI67" s="26"/>
-      <c r="ACJ67" s="26"/>
-      <c r="ACK67" s="26"/>
-      <c r="ACL67" s="26"/>
-      <c r="ACM67" s="26"/>
-      <c r="ACN67" s="26"/>
-      <c r="ACO67" s="26"/>
-      <c r="ACP67" s="26"/>
-      <c r="ACQ67" s="26"/>
-      <c r="ACR67" s="26"/>
-      <c r="ACS67" s="26"/>
-      <c r="ACT67" s="26"/>
-      <c r="ACU67" s="26"/>
-      <c r="ACV67" s="26"/>
-      <c r="ACW67" s="26"/>
-      <c r="ACX67" s="26"/>
-      <c r="ACY67" s="26"/>
-      <c r="ACZ67" s="26"/>
-      <c r="ADA67" s="26"/>
-      <c r="ADB67" s="26"/>
-      <c r="ADC67" s="26"/>
-      <c r="ADD67" s="26"/>
-      <c r="ADE67" s="26"/>
-      <c r="ADF67" s="26"/>
-      <c r="ADG67" s="26"/>
-      <c r="ADH67" s="26"/>
-      <c r="ADI67" s="26"/>
-      <c r="ADJ67" s="26"/>
-      <c r="ADK67" s="26"/>
-      <c r="ADL67" s="26"/>
-      <c r="ADM67" s="26"/>
-      <c r="ADN67" s="26"/>
-      <c r="ADO67" s="26"/>
-      <c r="ADP67" s="26"/>
-      <c r="ADQ67" s="26"/>
-      <c r="ADR67" s="26"/>
-      <c r="ADS67" s="26"/>
-      <c r="ADT67" s="26"/>
-      <c r="ADU67" s="26"/>
-      <c r="ADV67" s="26"/>
-      <c r="ADW67" s="26"/>
-      <c r="ADX67" s="26"/>
-      <c r="ADY67" s="26"/>
-      <c r="ADZ67" s="26"/>
-      <c r="AEA67" s="26"/>
-      <c r="AEB67" s="26"/>
-      <c r="AEC67" s="26"/>
-      <c r="AED67" s="26"/>
-      <c r="AEE67" s="26"/>
-      <c r="AEF67" s="26"/>
-      <c r="AEG67" s="26"/>
-      <c r="AEH67" s="26"/>
-      <c r="AEI67" s="26"/>
-      <c r="AEJ67" s="26"/>
-      <c r="AEK67" s="26"/>
-      <c r="AEL67" s="26"/>
-      <c r="AEM67" s="26"/>
-      <c r="AEN67" s="26"/>
-      <c r="AEO67" s="26"/>
-      <c r="AEP67" s="26"/>
-      <c r="AEQ67" s="26"/>
-      <c r="AER67" s="26"/>
-      <c r="AES67" s="26"/>
-      <c r="AET67" s="26"/>
-      <c r="AEU67" s="26"/>
-      <c r="AEV67" s="26"/>
-      <c r="AEW67" s="26"/>
-      <c r="AEX67" s="26"/>
-      <c r="AEY67" s="26"/>
-      <c r="AEZ67" s="26"/>
-      <c r="AFA67" s="26"/>
-      <c r="AFB67" s="26"/>
-      <c r="AFC67" s="26"/>
-      <c r="AFD67" s="26"/>
-      <c r="AFE67" s="26"/>
-      <c r="AFF67" s="26"/>
-      <c r="AFG67" s="26"/>
-      <c r="AFH67" s="26"/>
-      <c r="AFI67" s="26"/>
-      <c r="AFJ67" s="26"/>
-      <c r="AFK67" s="26"/>
-      <c r="AFL67" s="26"/>
-      <c r="AFM67" s="26"/>
-      <c r="AFN67" s="26"/>
-      <c r="AFO67" s="26"/>
-      <c r="AFP67" s="26"/>
-      <c r="AFQ67" s="26"/>
-      <c r="AFR67" s="26"/>
-      <c r="AFS67" s="26"/>
-      <c r="AFT67" s="26"/>
-      <c r="AFU67" s="26"/>
-      <c r="AFV67" s="26"/>
-      <c r="AFW67" s="26"/>
-      <c r="AFX67" s="26"/>
-      <c r="AFY67" s="26"/>
-      <c r="AFZ67" s="26"/>
-      <c r="AGA67" s="26"/>
-      <c r="AGB67" s="26"/>
-      <c r="AGC67" s="26"/>
-      <c r="AGD67" s="26"/>
-      <c r="AGE67" s="26"/>
-      <c r="AGF67" s="26"/>
-      <c r="AGG67" s="26"/>
-      <c r="AGH67" s="26"/>
-      <c r="AGI67" s="26"/>
-      <c r="AGJ67" s="26"/>
-      <c r="AGK67" s="26"/>
-      <c r="AGL67" s="26"/>
-      <c r="AGM67" s="26"/>
-      <c r="AGN67" s="26"/>
-      <c r="AGO67" s="26"/>
-      <c r="AGP67" s="26"/>
-      <c r="AGQ67" s="26"/>
-      <c r="AGR67" s="26"/>
-      <c r="AGS67" s="26"/>
-      <c r="AGT67" s="26"/>
-      <c r="AGU67" s="26"/>
-      <c r="AGV67" s="26"/>
-      <c r="AGW67" s="26"/>
-      <c r="AGX67" s="26"/>
-      <c r="AGY67" s="26"/>
-      <c r="AGZ67" s="26"/>
-      <c r="AHA67" s="26"/>
-      <c r="AHB67" s="26"/>
-      <c r="AHC67" s="26"/>
-      <c r="AHD67" s="26"/>
-      <c r="AHE67" s="26"/>
-      <c r="AHF67" s="26"/>
-      <c r="AHG67" s="26"/>
-      <c r="AHH67" s="26"/>
-      <c r="AHI67" s="26"/>
-      <c r="AHJ67" s="26"/>
-      <c r="AHK67" s="26"/>
-      <c r="AHL67" s="26"/>
-      <c r="AHM67" s="26"/>
-      <c r="AHN67" s="26"/>
-      <c r="AHO67" s="26"/>
-      <c r="AHP67" s="26"/>
-      <c r="AHQ67" s="26"/>
-      <c r="AHR67" s="26"/>
-      <c r="AHS67" s="26"/>
-      <c r="AHT67" s="26"/>
-      <c r="AHU67" s="26"/>
-      <c r="AHV67" s="26"/>
-      <c r="AHW67" s="26"/>
-      <c r="AHX67" s="26"/>
-      <c r="AHY67" s="26"/>
-      <c r="AHZ67" s="26"/>
-      <c r="AIA67" s="26"/>
-      <c r="AIB67" s="26"/>
-      <c r="AIC67" s="26"/>
-      <c r="AID67" s="26"/>
-      <c r="AIE67" s="26"/>
-      <c r="AIF67" s="26"/>
-      <c r="AIG67" s="26"/>
-      <c r="AIH67" s="26"/>
-      <c r="AII67" s="26"/>
-      <c r="AIJ67" s="26"/>
-      <c r="AIK67" s="26"/>
-      <c r="AIL67" s="26"/>
-      <c r="AIM67" s="26"/>
-      <c r="AIN67" s="26"/>
-      <c r="AIO67" s="26"/>
-      <c r="AIP67" s="26"/>
-      <c r="AIQ67" s="26"/>
-      <c r="AIR67" s="26"/>
-      <c r="AIS67" s="26"/>
-      <c r="AIT67" s="26"/>
-      <c r="AIU67" s="26"/>
-      <c r="AIV67" s="26"/>
-      <c r="AIW67" s="26"/>
-      <c r="AIX67" s="26"/>
-      <c r="AIY67" s="26"/>
-      <c r="AIZ67" s="26"/>
-      <c r="AJA67" s="26"/>
-      <c r="AJB67" s="26"/>
-      <c r="AJC67" s="26"/>
-      <c r="AJD67" s="26"/>
-      <c r="AJE67" s="26"/>
-      <c r="AJF67" s="26"/>
-      <c r="AJG67" s="26"/>
-      <c r="AJH67" s="26"/>
-      <c r="AJI67" s="26"/>
-      <c r="AJJ67" s="26"/>
-      <c r="AJK67" s="26"/>
-      <c r="AJL67" s="26"/>
-      <c r="AJM67" s="26"/>
-      <c r="AJN67" s="26"/>
-      <c r="AJO67" s="26"/>
-      <c r="AJP67" s="26"/>
-      <c r="AJQ67" s="26"/>
-      <c r="AJR67" s="26"/>
-      <c r="AJS67" s="26"/>
-      <c r="AJT67" s="26"/>
-      <c r="AJU67" s="26"/>
-      <c r="AJV67" s="26"/>
-      <c r="AJW67" s="26"/>
-      <c r="AJX67" s="26"/>
-      <c r="AJY67" s="26"/>
-      <c r="AJZ67" s="26"/>
-      <c r="AKA67" s="26"/>
-      <c r="AKB67" s="26"/>
-      <c r="AKC67" s="26"/>
-      <c r="AKD67" s="26"/>
-      <c r="AKE67" s="26"/>
-      <c r="AKF67" s="26"/>
-      <c r="AKG67" s="26"/>
-      <c r="AKH67" s="26"/>
-      <c r="AKI67" s="26"/>
-      <c r="AKJ67" s="26"/>
-      <c r="AKK67" s="26"/>
-      <c r="AKL67" s="26"/>
-      <c r="AKM67" s="26"/>
-      <c r="AKN67" s="26"/>
-      <c r="AKO67" s="26"/>
-      <c r="AKP67" s="26"/>
-      <c r="AKQ67" s="26"/>
-      <c r="AKR67" s="26"/>
-      <c r="AKS67" s="26"/>
-      <c r="AKT67" s="26"/>
-      <c r="AKU67" s="26"/>
-      <c r="AKV67" s="26"/>
-      <c r="AKW67" s="26"/>
-      <c r="AKX67" s="26"/>
-      <c r="AKY67" s="26"/>
-      <c r="AKZ67" s="26"/>
-      <c r="ALA67" s="26"/>
-      <c r="ALB67" s="26"/>
-      <c r="ALC67" s="26"/>
-      <c r="ALD67" s="26"/>
-      <c r="ALE67" s="26"/>
-      <c r="ALF67" s="26"/>
-      <c r="ALG67" s="26"/>
-      <c r="ALH67" s="26"/>
-      <c r="ALI67" s="26"/>
-      <c r="ALJ67" s="26"/>
-      <c r="ALK67" s="26"/>
-      <c r="ALL67" s="26"/>
-      <c r="ALM67" s="26"/>
-      <c r="ALN67" s="26"/>
-      <c r="ALO67" s="26"/>
-      <c r="ALP67" s="26"/>
-      <c r="ALQ67" s="26"/>
-      <c r="ALR67" s="26"/>
-      <c r="ALS67" s="26"/>
-      <c r="ALT67" s="26"/>
-      <c r="ALU67" s="26"/>
-      <c r="ALV67" s="26"/>
-      <c r="ALW67" s="26"/>
-      <c r="ALX67" s="26"/>
-      <c r="ALY67" s="26"/>
-      <c r="ALZ67" s="26"/>
-      <c r="AMA67" s="26"/>
-      <c r="AMB67" s="26"/>
-      <c r="AMC67" s="26"/>
-      <c r="AMD67" s="26"/>
-      <c r="AME67" s="26"/>
-      <c r="AMF67" s="26"/>
-      <c r="AMG67" s="26"/>
-      <c r="AMH67" s="26"/>
-      <c r="AMI67" s="26"/>
-      <c r="AMJ67" s="26"/>
-      <c r="AMK67" s="26"/>
-    </row>
-    <row r="68" spans="1:1025" x14ac:dyDescent="0.2">
-      <c r="B68" s="35" t="s">
+      <c r="C67" s="32"/>
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B68" s="33" t="s">
         <v>220</v>
       </c>
-      <c r="C68" s="35"/>
+      <c r="C68" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -7481,16 +4447,16 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="5" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
     </row>
     <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="35" t="s">
         <v>196</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -7501,7 +4467,7 @@
       <c r="F6" s="8"/>
     </row>
     <row r="7" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="37"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="8" t="s">
         <v>198</v>
       </c>
@@ -7510,7 +4476,7 @@
       <c r="F7" s="8"/>
     </row>
     <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="37"/>
+      <c r="B8" s="35"/>
       <c r="C8" s="8" t="s">
         <v>199</v>
       </c>
@@ -7519,7 +4485,7 @@
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="37"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="8" t="s">
         <v>200</v>
       </c>
@@ -7528,13 +4494,13 @@
       <c r="F9" s="8"/>
     </row>
     <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="37"/>
-      <c r="C10" s="38" t="s">
+      <c r="B10" s="35"/>
+      <c r="C10" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7554,7 +4520,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B1:D17"/>
+  <dimension ref="B1:D18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.6640625" customWidth="1"/>
@@ -7564,11 +4530,11 @@
   <sheetData>
     <row r="1" spans="2:4" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="41"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="39"/>
     </row>
     <row r="3" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="11" t="s">
@@ -7724,14 +4690,25 @@
         <v>224</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="B17" s="20" t="s">
+    <row r="17" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B17" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>268</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="B18" s="20" t="s">
         <v>287</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C18" s="21" t="s">
         <v>288</v>
       </c>
-      <c r="D17" s="22" t="s">
+      <c r="D18" s="22" t="s">
         <v>289</v>
       </c>
     </row>

</xml_diff>